<commit_message>
Element list: state the registered namespace instead of placeholder
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -482,7 +482,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>version 0.9 (draft, placeholder namespace)</t>
+          <t>version 0.9, namespace https://w3id.org/euonair/course#</t>
         </is>
       </c>
     </row>
@@ -9922,7 +9922,7 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Offered by schema.org for the licence of the structured data, whatever vocabularies it combines. Decided with the review and publication of the profile (Section 10); openly published records should state it.</t>
+          <t>Offered by schema.org for the licence of the structured data, whatever vocabularies it combines. Decided with the review of the profile (Section 10); openly published records should state it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Element list: label design input by the requirements of the MS4 report
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -1724,7 +1724,7 @@
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 10/10; manual course-specific ●6/10; WP4 Md 5, 90 %, ✔ · P3 T2, T3, T4, T7, T8, T10; concept, MyAI University</t>
+          <t>P1 ✓3 · P2 10/10; manual course-specific ●6/10; WP4 Md 5, 90 %, ✔ · P3 T2, T3, T4, T7, T8, T10; design input, MyAI University</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
-          <t>P1 hook · P2 0/10 (no Bloom tagging in any document) · P3 T3, T8, T10; concept, MyAI University</t>
+          <t>P1 hook · P2 0/10 (no Bloom tagging in any document) · P3 T3, T8, T10; design input, MyAI University</t>
         </is>
       </c>
       <c r="S20" s="3" t="inlineStr">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="R21" s="3" t="inlineStr">
         <is>
-          <t>P1 hook · P2 manual ●2/10, ◐4/10 (five different outcome models in use) · P3 T10; concept</t>
+          <t>P1 hook · P2 manual ●2/10, ◐4/10 (five different outcome models in use) · P3 T10; design input</t>
         </is>
       </c>
       <c r="S21" s="3" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="R23" s="3" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 competences assessed 1/10 (+3); manual ●2/10; WP4 Md 5, 80 %, ✔ · P3 T4, T8, T12; WP4: structured outcome–assessment mapping for most courses 3/11, for some 2/11; concept</t>
+          <t>P1 ✓2 · P2 competences assessed 1/10 (+3); manual ●2/10; WP4 Md 5, 80 %, ✔ · P3 T4, T8, T12; WP4: structured outcome–assessment mapping for most courses 3/11, for some 2/11; design input</t>
         </is>
       </c>
       <c r="S23" s="3" t="inlineStr">
@@ -2888,7 +2888,7 @@
       </c>
       <c r="R24" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 n.m. (field present only in one blank template); named as missing in WP4 · P3 T7, T9; concept</t>
+          <t>P1 ✗ · P2 n.m. (field present only in one blank template); named as missing in WP4 · P3 T7, T9; design input</t>
         </is>
       </c>
       <c r="S24" s="3" t="inlineStr">
@@ -3082,7 +3082,7 @@
       </c>
       <c r="R26" s="3" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 manual: prior knowledge as a field of its own (prose) at 1 partner; competences as structured items only in 1 blank template · P3 T2, T5; concept, MyAI University</t>
+          <t>P1 ✓3 · P2 manual: prior knowledge as a field of its own (prose) at 1 partner; competences as structured items only in 1 blank template · P3 T2, T5; design input, MyAI University</t>
         </is>
       </c>
       <c r="S26" s="3" t="inlineStr">
@@ -3276,7 +3276,7 @@
       </c>
       <c r="R28" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 n.m. (no field in any partner document) · P3 T2, T3; concept</t>
+          <t>P1 ✗ · P2 n.m. (no field in any partner document) · P3 T2, T3; design input</t>
         </is>
       </c>
       <c r="S28" s="3" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="R30" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 no field in any partner; AI rules found only at assessment level (A12) · P3 A1, T3; all reported institutional policies PDF/web only; concept</t>
+          <t>P1 ✗ · P2 no field in any partner; AI rules found only at assessment level (A12) · P3 A1, T3; all reported institutional policies PDF/web only; design input</t>
         </is>
       </c>
       <c r="S30" s="3" t="inlineStr">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="R31" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 1/10 (permitted aids of individual exams, 7 of 125 module descriptions) · P3 A1, A2, T9; institutional policies cover assessments at 7 of 9; concept</t>
+          <t>P1 ✗ · P2 1/10 (permitted aids of individual exams, 7 of 125 module descriptions) · P3 A1, A2, T9; institutional policies cover assessments at 7 of 9; design input</t>
         </is>
       </c>
       <c r="S31" s="3" t="inlineStr">
@@ -7738,7 +7738,7 @@
       </c>
       <c r="R74" s="5" t="inlineStr">
         <is>
-          <t>P1 hook · P2 n.m. · P3 A3; concept</t>
+          <t>P1 hook · P2 n.m. · P3 A3; design input</t>
         </is>
       </c>
       <c r="S74" s="5" t="inlineStr">
@@ -9126,7 +9126,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>ECTS "planned learning activities"; coded lists at 2/10 partners; concept-work formats</t>
+          <t>ECTS "planned learning activities"; coded lists at 2/10 partners; common teaching formats</t>
         </is>
       </c>
     </row>
@@ -9143,7 +9143,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>concept-work assessment types; partner verification-method lists (extensible)</t>
+          <t>common assessment types; partner verification-method lists (extensible)</t>
         </is>
       </c>
     </row>
@@ -9950,7 +9950,7 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="36" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="32.8" customWidth="1" min="11" max="11"/>
     <col width="9.600000000000001" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
     <col width="60" customWidth="1" min="14" max="14"/>
@@ -9962,7 +9962,7 @@
     <col width="10.4" customWidth="1" min="20" max="20"/>
     <col width="11.2" customWidth="1" min="21" max="21"/>
     <col width="8" customWidth="1" min="22" max="22"/>
-    <col width="9.600000000000001" customWidth="1" min="23" max="23"/>
+    <col width="13.6" customWidth="1" min="23" max="23"/>
     <col width="8" customWidth="1" min="24" max="24"/>
     <col width="8" customWidth="1" min="25" max="25"/>
   </cols>
@@ -10020,7 +10020,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>p3_concept</t>
+          <t>p3_design_input</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -10080,7 +10080,7 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>m_p3_concept</t>
+          <t>m_p3_design_input</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -13208,7 +13208,7 @@
       </c>
       <c r="K29" s="7" t="inlineStr">
         <is>
-          <t>MS4, MyAI University</t>
+          <t>requirements (Section 2), MyAI University</t>
         </is>
       </c>
       <c r="L29" s="7" t="inlineStr">
@@ -13329,7 +13329,7 @@
       </c>
       <c r="K30" s="7" t="inlineStr">
         <is>
-          <t>MS4</t>
+          <t>requirements (Section 2)</t>
         </is>
       </c>
       <c r="L30" s="7" t="inlineStr">
@@ -16053,7 +16053,7 @@
       </c>
       <c r="K54" s="7" t="inlineStr">
         <is>
-          <t>MS4</t>
+          <t>requirements (Section 2)</t>
         </is>
       </c>
       <c r="L54" s="7" t="inlineStr">
@@ -17357,7 +17357,7 @@
       </c>
       <c r="K66" s="7" t="inlineStr">
         <is>
-          <t>MS4, MyAI University</t>
+          <t>requirements (Section 2), MyAI University</t>
         </is>
       </c>
       <c r="L66" s="7" t="inlineStr">
@@ -17472,7 +17472,7 @@
       </c>
       <c r="K67" s="7" t="inlineStr">
         <is>
-          <t>MS4</t>
+          <t>requirements (Section 2)</t>
         </is>
       </c>
       <c r="L67" s="7" t="inlineStr">
@@ -17698,7 +17698,7 @@
       </c>
       <c r="K69" s="7" t="inlineStr">
         <is>
-          <t>MS4</t>
+          <t>requirements (Section 2)</t>
         </is>
       </c>
       <c r="L69" s="7" t="inlineStr">
@@ -17809,7 +17809,7 @@
       </c>
       <c r="K70" s="7" t="inlineStr">
         <is>
-          <t>MS4, MyAI University</t>
+          <t>requirements (Section 2), MyAI University</t>
         </is>
       </c>
       <c r="L70" s="7" t="inlineStr">
@@ -17924,7 +17924,7 @@
       </c>
       <c r="K71" s="7" t="inlineStr">
         <is>
-          <t>MS4</t>
+          <t>requirements (Section 2)</t>
         </is>
       </c>
       <c r="L71" s="7" t="inlineStr">
@@ -18035,7 +18035,7 @@
       </c>
       <c r="K72" s="7" t="inlineStr">
         <is>
-          <t>MS4</t>
+          <t>requirements (Section 2)</t>
         </is>
       </c>
       <c r="L72" s="7" t="inlineStr">
@@ -18146,7 +18146,7 @@
       </c>
       <c r="K73" s="7" t="inlineStr">
         <is>
-          <t>MS4</t>
+          <t>requirements (Section 2)</t>
         </is>
       </c>
       <c r="L73" s="7" t="inlineStr">
@@ -18360,7 +18360,7 @@
       <c r="J75" s="7" t="inlineStr"/>
       <c r="K75" s="7" t="inlineStr">
         <is>
-          <t>MS4 (could)</t>
+          <t>requirements (optional)</t>
         </is>
       </c>
       <c r="L75" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Element list: ELM mappings checked against ELM 3.3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -561,7 +561,7 @@
     <col width="58.40000000000001" customWidth="1" min="11" max="11"/>
     <col width="19.2" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
-    <col width="41.6" customWidth="1" min="14" max="14"/>
+    <col width="44" customWidth="1" min="14" max="14"/>
     <col width="60" customWidth="1" min="15" max="15"/>
     <col width="56.8" customWidth="1" min="16" max="16"/>
     <col width="36" customWidth="1" min="17" max="17"/>
@@ -928,7 +928,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>≈ LAS type</t>
+          <t>≈ LAS dcType</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>LOpp providedBy; LAS ≈ awardedBy</t>
+          <t>LOpp providedBy; LAS awardingOpportunity → awardingBody</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>LAS EQFLevel, NQFLevel</t>
+          <t>LAS educationLevel (EQF / NQF concept)</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="N21" s="3" t="inlineStr">
         <is>
-          <t>≈ LOut type</t>
+          <t>≈ LOut dcType</t>
         </is>
       </c>
       <c r="O21" s="3" t="inlineStr">
@@ -3838,7 +3838,7 @@
       </c>
       <c r="N34" s="4" t="inlineStr">
         <is>
-          <t>LAS alternativeLabel</t>
+          <t>LAS altLabel</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
@@ -5002,7 +5002,7 @@
       </c>
       <c r="N46" s="4" t="inlineStr">
         <is>
-          <t>≈ Organisation (sub-unit)</t>
+          <t>Organisation subOrganizationOf / hasSubOrganization</t>
         </is>
       </c>
       <c r="O46" s="4" t="inlineStr">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="N75" s="5" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>≈ LAS status</t>
         </is>
       </c>
       <c r="O75" s="5" t="inlineStr">
@@ -8529,7 +8529,7 @@
       </c>
       <c r="N3" s="6" t="inlineStr">
         <is>
-          <t>≈ LActS directedBy</t>
+          <t>≈ LearningActivity directedBy</t>
         </is>
       </c>
       <c r="O3" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Element list and pages: wording from the final report review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -7984,7 +7984,7 @@
       </c>
       <c r="I77" s="5" t="inlineStr">
         <is>
-          <t>maintainer (≈ sdPublisher); maintainer, editor</t>
+          <t>maintainer (≈ sdPublisher)</t>
         </is>
       </c>
       <c r="J77" s="5" t="inlineStr">
@@ -9790,7 +9790,7 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>MoSCoW "Could"; no evidence collected. Candidate for D2.2/D4.2.</t>
+          <t>Low priority in the requirements; candidate for D2.2/D4.2.</t>
         </is>
       </c>
     </row>
@@ -9856,7 +9856,7 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Practised by 2/10 partners. Professional relevance is covered by X34.</t>
+          <t>Practised by 2/10 partners. A sustainability focus can be stated in the content description (C06) or as a keyword (X03).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Validator, term index and policy rules; profile fixes from review
- validate.py with the pinned schema.org context: 59 offline tests
  (positive examples, negative variants, JSON Schema and SHACL agreement)
- Landing page: entry for every euonair: term used, conventions and
  AI-use policy precedence rules
- Schema and shapes: EQF plus optional NQF levels, closed vocabularies
  checked by value, exclusive weight alternatives, IRI links
- Element list: Sources sheet resolving source codes to references

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vocabularies" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not included" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate fields" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -494,7 +495,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Elements (core, extensions, record) · Linked offering · Vocabularies · Not included · Candidate fields</t>
+          <t>Elements (core, extensions, record) · Linked offering · Vocabularies · Not included · Candidate fields · Sources (key to the source codes in Candidate fields)</t>
         </is>
       </c>
     </row>
@@ -851,7 +852,7 @@
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓5 · P2 10/10; WP4 Md 5, 82 %, ✔ · P3 A3, T5; MyAI University</t>
+          <t>P1 ✓5 · P2 10/10; WP4 Md 5, 82 %, ✔ · P3 A3; MyAI University</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
@@ -948,7 +949,7 @@
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 2/10 (combined field only; +3 from structure); WP4 Md 4, 91 %, ✔ · P3 T5</t>
+          <t>P1 ✓3 · P2 2/10 (combined field only; +3 from structure); WP4 Md 4, 91 %, ✔ · P3 –</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
@@ -990,7 +991,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Ref → Organization (IRI, name, country as address/addressCountry, ISO 3166-1 alpha-2) 1..1</t>
+          <t>Ref → Organization (IRI, name, country: address.addressCountry, ISO 3166-1 alpha-2) 1..1</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1045,7 +1046,7 @@
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓4 · P2 3/10 (+2); WP4 Md 4, 64 %, ✘ · P3 T5; MyAI University</t>
+          <t>P1 ✓4 · P2 3/10 (+2); WP4 Md 4, 64 %, ✘ · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
@@ -1239,7 +1240,7 @@
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓5 · P2 10/10; WP4 Md 5, 100 %, ✔ · P3 T1, T2, T7; MyAI University</t>
+          <t>P1 ✓5 · P2 10/10; WP4 Md 5, 100 %, ✔ · P3 T1, T2, T5, T7; MyAI University</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
@@ -1336,7 +1337,7 @@
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 6/10 (+3); WP4 Md 4, 100 %, ✔ · P3 T1, T2, T7, T8</t>
+          <t>P1 ✓2 · P2 6/10 (+3); WP4 Md 4, 100 %, ✔ · P3 T1, T2, T5, T7, T8</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
@@ -1433,7 +1434,7 @@
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓5 · P2 7/10 (+2); WP4 Md 4, 55 %, ✘ · P3 T5, T6; MyAI University</t>
+          <t>P1 ✓5 · P2 7/10 (+2); WP4 Md 4, 55 %, ✘ · P3 T6; MyAI University</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
@@ -1470,12 +1471,12 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>EQF level of the unit (ECTS cycle derivable). National framework levels may be added.</t>
+          <t>EQF level of the unit (ECTS cycle derivable), given exactly once. National framework (NQF) levels may be added as further values of the same property.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Concept 1..1 (EQF IRI); NQF Concept 0..*</t>
+          <t>Concept 1..*: exactly one EQF IRI, plus NQF Concepts 0..*</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1500,7 +1501,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>1..1 0..*</t>
+          <t>1..* 0..*</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1530,7 +1531,7 @@
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓4 · P2 4/10 (+4); WP4 Md 4, 70 %, ✘ · P3 T1, T2, T10, T5; MyAI University</t>
+          <t>P1 ✓4 · P2 4/10 (+4); WP4 Md 4, 70 %, ✘ · P3 T1, T2, T5, T10; MyAI University</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
@@ -1627,7 +1628,7 @@
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 10/10; WP4 Md 4.5, 90 %, ✔ · P3 T7, T5, T11; MyAI University</t>
+          <t>P1 ✓3 · P2 10/10; WP4 Md 4.5, 90 %, ✔ · P3 T7, T11; MyAI University</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
@@ -1724,7 +1725,7 @@
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 10/10; manual course-specific ●6/10; WP4 Md 5, 90 %, ✔ · P3 T2, T3, T4, T7, T8, T10; design input, MyAI University</t>
+          <t>P1 ✓3 · P2 10/10; manual course-specific ●6/10; WP4 Md 5, 90 %, ✔ · P3 T2, T3, T4, T5, T7, T8, T10; design input, MyAI University</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
@@ -1821,7 +1822,7 @@
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 8/10; WP4 Md 4, 80 %, ✔ · P3 T5, T11; MyAI University</t>
+          <t>P1 ✓3 · P2 8/10; WP4 Md 4, 80 %, ✔ · P3 T11; MyAI University</t>
         </is>
       </c>
       <c r="S13" s="2" t="inlineStr">
@@ -1918,7 +1919,7 @@
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 9/10; WP4 Md 4, 90 %, ✔ · P3 T7, T5; MyAI University</t>
+          <t>P1 ✓3 · P2 9/10; WP4 Md 4, 90 %, ✔ · P3 T7; MyAI University</t>
         </is>
       </c>
       <c r="S14" s="2" t="inlineStr">
@@ -2112,7 +2113,7 @@
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓4 · P2 9/10 (+1); WP4 Md 4, 80 %, ✔ · P3 T7, T9; MyAI University</t>
+          <t>P1 ✓4 · P2 9/10 (+1); WP4 Md 4, 80 %, ✔ · P3 T5, T7, T9; MyAI University</t>
         </is>
       </c>
       <c r="S16" s="2" t="inlineStr">
@@ -2149,7 +2150,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Each graded or required assessment element. Mandatory sub-fields: method; weight (%) or weight range (min–max); group mode (individual / group / mixed). Optional: name, duration in minutes, ECTS share. Required ungraded components carry weight 0. Ranges: min ≤ max and Σmin ≤ 100 ≤ Σmax; an offering's final weight refers to the same component (euonair:specifiedBy).</t>
+          <t>Each graded or required assessment element. Mandatory sub-fields: method; weight (%) or weight range (min–max); group mode (individual / group / mixed). Optional: name, duration in minutes, ECTS share. The weight is the component's contribution to the numerical grade of the unit. Where the unit has a numerical grade, the weights of the graded components sum to 100; ranges of graded components satisfy min ≤ max and Σmin ≤ 100 ≤ Σmax. Required ungraded (pass/fail) components carry weight 0 and are recorded as completion requirements. For a unit graded pass/fail as a whole (C16), no weight total applies. An offering's final weight refers to the same component (euonair:specifiedBy).</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -2246,7 +2247,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Whether the unit is graded or pass/fail, plus a reference to the grading scale.</t>
+          <t>Whether the unit is graded or pass/fail, plus a reference to the grading scale. In a unit graded pass/fail as a whole, all components are completion requirements with weight 0, and no weight total applies (C15).</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2500,7 +2501,7 @@
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
-          <t>P1 hook · P2 0/10 (no Bloom tagging in any document) · P3 T3, T8, T10; design input, MyAI University</t>
+          <t>P1 hook · P2 0/10 (no Bloom tagging in any document) · P3 T3, T5, T8, T10; design input, MyAI University</t>
         </is>
       </c>
       <c r="S20" s="3" t="inlineStr">
@@ -2791,7 +2792,7 @@
       </c>
       <c r="R23" s="3" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 competences assessed 1/10 (+3); manual ●2/10; WP4 Md 5, 80 %, ✔ · P3 T4, T8, T12; WP4: structured outcome–assessment mapping for most courses 3/11, for some 2/11; design input</t>
+          <t>P1 ✓2 · P2 competences assessed 1/10 (+3); manual ●2/10; WP4 Md 5, 80 %, ✔ · P3 T4, T5, T8, T12; WP4: structured outcome–assessment mapping for most courses 3/11, for some 2/11; design input</t>
         </is>
       </c>
       <c r="S23" s="3" t="inlineStr">
@@ -2888,7 +2889,7 @@
       </c>
       <c r="R24" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 n.m. (field present only in one blank template); named as missing in WP4 · P3 T7, T9; design input</t>
+          <t>P1 ✗ · P2 n.m. (field present only in one blank template); named as missing in WP4 · P3 T5, T7, T9; design input</t>
         </is>
       </c>
       <c r="S24" s="3" t="inlineStr">
@@ -3470,7 +3471,7 @@
       </c>
       <c r="R30" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 no field in any partner; AI rules found only at assessment level (A12) · P3 A1, T3; all reported institutional policies PDF/web only; design input</t>
+          <t>P1 ✗ · P2 no field in any partner; AI rules found only at assessment level (A12) · P3 T3, A1; all reported institutional policies PDF/web only; design input</t>
         </is>
       </c>
       <c r="S30" s="3" t="inlineStr">
@@ -3567,7 +3568,7 @@
       </c>
       <c r="R31" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 1/10 (permitted aids of individual exams, 7 of 125 module descriptions) · P3 A1, A2, T9; institutional policies cover assessments at 7 of 9; design input</t>
+          <t>P1 ✗ · P2 1/10 (permitted aids of individual exams, 7 of 125 module descriptions) · P3 T9, A1, A2; institutional policies cover assessments at 7 of 9; design input</t>
         </is>
       </c>
       <c r="S31" s="3" t="inlineStr">
@@ -3664,7 +3665,7 @@
       </c>
       <c r="R32" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 n.m.; exam settings implicit in assessment methods · P3 A1, T4; Corbin et al., 2025; Verbeken et al., 2026 (supervised setting rated low risk in an institutional rubric)</t>
+          <t>P1 ✗ · P2 n.m.; exam settings implicit in assessment methods · P3 T4, A1; Corbin et al., 2025; Verbeken et al., 2026 (supervised setting rated low risk in an institutional rubric)</t>
         </is>
       </c>
       <c r="S32" s="3" t="inlineStr">
@@ -3955,7 +3956,7 @@
       </c>
       <c r="R35" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 n.m.; WP4 via merged item · P3 T5; MyAI University</t>
+          <t>P1 ✓2 · P2 n.m.; WP4 via merged item · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S35" s="4" t="inlineStr">
@@ -4052,7 +4053,7 @@
       </c>
       <c r="R36" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 0/10; WP4 Md 4, 64 %, ✘ · P3 T5; MyAI University</t>
+          <t>P1 ✓3 · P2 0/10; WP4 Md 4, 64 %, ✘ · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S36" s="4" t="inlineStr">
@@ -4149,7 +4150,7 @@
       </c>
       <c r="R37" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓5 · P2 0/10 (+2 at programme level); WP4 Md 3, 36 %, ✘ · P3 T5; MyAI University</t>
+          <t>P1 ✓5 · P2 0/10 (+2 at programme level); WP4 Md 3, 36 %, ✘ · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S37" s="4" t="inlineStr">
@@ -4440,7 +4441,7 @@
       </c>
       <c r="R40" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 0/10; WP4 Md 4, 60 %, ✘ · P3 T10, T5; MyAI University</t>
+          <t>P1 ✓3 · P2 0/10; WP4 Md 4, 60 %, ✘ · P3 T10; MyAI University</t>
         </is>
       </c>
       <c r="S40" s="4" t="inlineStr">
@@ -4537,7 +4538,7 @@
       </c>
       <c r="R41" s="4" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 n.m. (AI appears as subject matter at ≥4/10 partners, free text) · P3 T5; MyAI University</t>
+          <t>P1 ✗ · P2 n.m. (AI appears as subject matter at ≥4/10 partners, free text) · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S41" s="4" t="inlineStr">
@@ -4731,7 +4732,7 @@
       </c>
       <c r="R43" s="4" t="inlineStr">
         <is>
-          <t>P1 ◐ (ECTS, programme level) · P2 2/10 (field inventory, outside the 39 fields) · P3 T5; MyAI University</t>
+          <t>P1 ◐ (ECTS, programme level) · P2 2/10 (field inventory, outside the 39 fields) · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S43" s="4" t="inlineStr">
@@ -4925,7 +4926,7 @@
       </c>
       <c r="R45" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 2/10 (+1); WP4 Md 4, 70 %, ✘ · P3 T5; MyAI University</t>
+          <t>P1 ✓2 · P2 2/10 (+1); WP4 Md 4, 70 %, ✘ · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S45" s="4" t="inlineStr">
@@ -5119,7 +5120,7 @@
       </c>
       <c r="R47" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓5 (programme) / ✓1 (obligation, position) · P2 position 6/10 (+3), compulsory/elective 3/10, track 3/10 (+3), parent programme 2/10 (+1); WP4 #6 Md 4, 73 %, ✘; #7 Md 4, 64 %, ✘; #8 Md 3, 45 %, ✘; #9 Md 4, 55 %, ✘ · P3 T5, T11</t>
+          <t>P1 ✓5 (programme) / ✓1 (obligation, position) · P2 position 6/10 (+3), compulsory/elective 3/10, track 3/10 (+3), parent programme 2/10 (+1); WP4 #6 Md 4, 73 %, ✘; #7 Md 4, 64 %, ✘; #8 Md 3, 45 %, ✘; #9 Md 4, 55 %, ✘ · P3 T11</t>
         </is>
       </c>
       <c r="S47" s="4" t="inlineStr">
@@ -5410,7 +5411,7 @@
       </c>
       <c r="R50" s="4" t="inlineStr">
         <is>
-          <t>P1 hook · P2 2/10; WP4 Md 4, 70 %, ✘ · P3 T5</t>
+          <t>P1 hook · P2 2/10; WP4 Md 4, 70 %, ✘ · P3 –</t>
         </is>
       </c>
       <c r="S50" s="4" t="inlineStr">
@@ -5507,7 +5508,7 @@
       </c>
       <c r="R51" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 n.m.; WP4 via merged item · P3 T5</t>
+          <t>P1 ✓2 · P2 n.m.; WP4 via merged item · P3 –</t>
         </is>
       </c>
       <c r="S51" s="4" t="inlineStr">
@@ -5604,7 +5605,7 @@
       </c>
       <c r="R52" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 1/10 (+2); WP4 Md 4, 70 %, ✘ · P3 T5; MyAI University</t>
+          <t>P1 ✓2 · P2 1/10 (+2); WP4 Md 4, 70 %, ✘ · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S52" s="4" t="inlineStr">
@@ -5701,7 +5702,7 @@
       </c>
       <c r="R53" s="4" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 n.m. · P3 T5; MyAI University</t>
+          <t>P1 ✗ · P2 n.m. · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S53" s="4" t="inlineStr">
@@ -5798,7 +5799,7 @@
       </c>
       <c r="R54" s="4" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 n.m. · P3 T5; MyAI University</t>
+          <t>P1 ✗ · P2 n.m. · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S54" s="4" t="inlineStr">
@@ -5895,7 +5896,7 @@
       </c>
       <c r="R55" s="4" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 n.m. · P3 T5; MyAI University</t>
+          <t>P1 ✗ · P2 n.m. · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S55" s="4" t="inlineStr">
@@ -6186,7 +6187,7 @@
       </c>
       <c r="R58" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 n.m. · P3 T5; MyAI University</t>
+          <t>P1 ✓2 · P2 n.m. · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S58" s="4" t="inlineStr">
@@ -6283,7 +6284,7 @@
       </c>
       <c r="R59" s="4" t="inlineStr">
         <is>
-          <t>P1 hook · P2 n.m. · P3 T5; MyAI University</t>
+          <t>P1 hook · P2 n.m. · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S59" s="4" t="inlineStr">
@@ -6380,7 +6381,7 @@
       </c>
       <c r="R60" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 1/10 (+4); WP4 Md 3, 45 %, ✘ · P3 T5; MyAI University</t>
+          <t>P1 ✓2 · P2 1/10 (+4); WP4 Md 3, 45 %, ✘ · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S60" s="4" t="inlineStr">
@@ -6477,7 +6478,7 @@
       </c>
       <c r="R61" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓1 · P2 0/10 (+2); WP4 Md 3, 45 %, ✘ · P3 T5; MyAI University</t>
+          <t>P1 ✓1 · P2 0/10 (+2); WP4 Md 3, 45 %, ✘ · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S61" s="4" t="inlineStr">
@@ -6574,7 +6575,7 @@
       </c>
       <c r="R62" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓1 · P2 n.m.; WP4 Md 3, 45 %, ✘ · P3 T5; MyAI University</t>
+          <t>P1 ✓1 · P2 n.m.; WP4 Md 3, 45 %, ✘ · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S62" s="4" t="inlineStr">
@@ -6671,7 +6672,7 @@
       </c>
       <c r="R63" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓1 · P2 n.m.; WP4 Md 3, 45 %, ✘ · P3 T5; MyAI University</t>
+          <t>P1 ✓1 · P2 n.m.; WP4 Md 3, 45 %, ✘ · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S63" s="4" t="inlineStr">
@@ -6865,7 +6866,7 @@
       </c>
       <c r="R65" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 2/10 (+6); WP4 Md 3.5, 50 %, ✘ · P3 T5; MyAI University</t>
+          <t>P1 ✓2 · P2 2/10 (+6); WP4 Md 3.5, 50 %, ✘ · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S65" s="4" t="inlineStr">
@@ -10360,7 +10361,7 @@
       <c r="I4" s="7" t="inlineStr"/>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>A3 More trust in AI output with visible sources (67 %); T5 Personalised learning recommendations (65 %)</t>
+          <t>A3 More trust in AI output with visible sources (67 %)</t>
         </is>
       </c>
       <c r="K4" s="7" t="inlineStr">
@@ -10695,11 +10696,7 @@
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr"/>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J7" s="7" t="inlineStr"/>
       <c r="K7" s="7" t="inlineStr"/>
       <c r="L7" s="7" t="inlineStr">
         <is>
@@ -10749,7 +10746,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -10808,11 +10805,7 @@
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr"/>
-      <c r="J8" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J8" s="7" t="inlineStr"/>
       <c r="K8" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -10866,7 +10859,7 @@
       </c>
       <c r="V8" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W8" s="7" t="inlineStr">
@@ -11030,11 +11023,7 @@
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr"/>
-      <c r="J10" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J10" s="7" t="inlineStr"/>
       <c r="K10" s="7" t="inlineStr"/>
       <c r="L10" s="7" t="inlineStr">
         <is>
@@ -11084,7 +11073,7 @@
       </c>
       <c r="V10" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W10" s="7" t="inlineStr">
@@ -11250,11 +11239,7 @@
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr"/>
-      <c r="J12" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J12" s="7" t="inlineStr"/>
       <c r="K12" s="7" t="inlineStr"/>
       <c r="L12" s="7" t="inlineStr">
         <is>
@@ -11304,7 +11289,7 @@
       </c>
       <c r="V12" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W12" s="7" t="inlineStr">
@@ -11365,7 +11350,7 @@
       <c r="I13" s="7" t="inlineStr"/>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>T5 Personalised learning recommendations (65 %); T11 Questions on regulations and procedures (61 %)</t>
+          <t>T11 Questions on regulations and procedures (61 %)</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr"/>
@@ -11476,11 +11461,7 @@
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr"/>
-      <c r="J14" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J14" s="7" t="inlineStr"/>
       <c r="K14" s="7" t="inlineStr"/>
       <c r="L14" s="7" t="inlineStr">
         <is>
@@ -11530,7 +11511,7 @@
       </c>
       <c r="V14" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W14" s="7" t="inlineStr">
@@ -11813,7 +11794,7 @@
       <c r="I17" s="7" t="inlineStr"/>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised learning recommendations (65 %)</t>
+          <t>T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised exercise and learning recommendations within a course (65 %)</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -11930,7 +11911,7 @@
       <c r="I18" s="7" t="inlineStr"/>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T7 Course outlines and lesson plans (64 %)</t>
+          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %)</t>
         </is>
       </c>
       <c r="K18" s="7" t="inlineStr">
@@ -12049,11 +12030,7 @@
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr"/>
-      <c r="J19" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J19" s="7" t="inlineStr"/>
       <c r="K19" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -12103,7 +12080,7 @@
       </c>
       <c r="V19" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W19" s="7" t="inlineStr">
@@ -12164,7 +12141,7 @@
       <c r="I20" s="7" t="inlineStr"/>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T7 Course outlines and lesson plans (64 %); T8 Quiz or exam questions (63 %)</t>
+          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %); T8 Quiz or exam questions (63 %)</t>
         </is>
       </c>
       <c r="K20" s="7" t="inlineStr"/>
@@ -12275,11 +12252,7 @@
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr"/>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J21" s="7" t="inlineStr"/>
       <c r="K21" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -12333,7 +12306,7 @@
       </c>
       <c r="V21" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W21" s="7" t="inlineStr">
@@ -12392,11 +12365,7 @@
         </is>
       </c>
       <c r="I22" s="7" t="inlineStr"/>
-      <c r="J22" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J22" s="7" t="inlineStr"/>
       <c r="K22" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -12450,7 +12419,7 @@
       </c>
       <c r="V22" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W22" s="7" t="inlineStr">
@@ -12511,7 +12480,7 @@
       <c r="I23" s="7" t="inlineStr"/>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>T5 Personalised learning recommendations (65 %); T6 Language learning or translation support (78 %)</t>
+          <t>T6 Language learning or translation support (78 %)</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
@@ -12739,11 +12708,7 @@
         </is>
       </c>
       <c r="I25" s="7" t="inlineStr"/>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J25" s="7" t="inlineStr"/>
       <c r="K25" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -12797,7 +12762,7 @@
       </c>
       <c r="V25" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W25" s="7" t="inlineStr">
@@ -12856,11 +12821,7 @@
         </is>
       </c>
       <c r="I26" s="7" t="inlineStr"/>
-      <c r="J26" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J26" s="7" t="inlineStr"/>
       <c r="K26" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -12914,7 +12875,7 @@
       </c>
       <c r="V26" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W26" s="7" t="inlineStr">
@@ -13203,7 +13164,7 @@
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>T2 Explanations of concepts (AI as tutor) (88 %); T3 Solving or explaining problems step by step (87 %); T4 Exam preparation (86 %); T7 Course outlines and lesson plans (64 %); T8 Quiz or exam questions (63 %); T10 Learning objectives and syllabi (52 %)</t>
+          <t>T2 Explanations of concepts (AI as tutor) (88 %); T3 Solving or explaining problems step by step (87 %); T4 Exam preparation (86 %); T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %); T8 Quiz or exam questions (63 %); T10 Learning objectives and syllabi (52 %)</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
@@ -13324,7 +13285,7 @@
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>T4 Exam preparation (86 %); T8 Quiz or exam questions (63 %); T12 Written feedback and grading rubrics (26 %)</t>
+          <t>T4 Exam preparation (86 %); T5 Personalised exercise and learning recommendations within a course (65 %); T8 Quiz or exam questions (63 %); T12 Written feedback and grading rubrics (26 %)</t>
         </is>
       </c>
       <c r="K30" s="7" t="inlineStr">
@@ -13441,7 +13402,7 @@
       <c r="I31" s="7" t="inlineStr"/>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>T10 Learning objectives and syllabi (52 %); T5 Personalised learning recommendations (65 %)</t>
+          <t>T10 Learning objectives and syllabi (52 %)</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
@@ -13558,7 +13519,7 @@
       <c r="I32" s="7" t="inlineStr"/>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T10 Learning objectives and syllabi (52 %); T5 Personalised learning recommendations (65 %)</t>
+          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T10 Learning objectives and syllabi (52 %); T5 Personalised exercise and learning recommendations within a course (65 %)</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
@@ -13671,7 +13632,7 @@
       <c r="I33" s="7" t="inlineStr"/>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised learning recommendations (65 %)</t>
+          <t>T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised exercise and learning recommendations within a course (65 %)</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
@@ -13788,7 +13749,7 @@
       <c r="I34" s="7" t="inlineStr"/>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>T5 Personalised learning recommendations (65 %); T11 Questions on regulations and procedures (61 %)</t>
+          <t>T11 Questions on regulations and procedures (61 %)</t>
         </is>
       </c>
       <c r="K34" s="7" t="inlineStr">
@@ -13903,11 +13864,7 @@
         </is>
       </c>
       <c r="I35" s="7" t="inlineStr"/>
-      <c r="J35" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J35" s="7" t="inlineStr"/>
       <c r="K35" s="7" t="inlineStr"/>
       <c r="L35" s="7" t="inlineStr">
         <is>
@@ -13953,7 +13910,7 @@
       </c>
       <c r="V35" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W35" s="7" t="inlineStr">
@@ -14014,7 +13971,7 @@
       <c r="I36" s="7" t="inlineStr"/>
       <c r="J36" s="7" t="inlineStr">
         <is>
-          <t>T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised learning recommendations (65 %)</t>
+          <t>T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised exercise and learning recommendations within a course (65 %)</t>
         </is>
       </c>
       <c r="K36" s="7" t="inlineStr">
@@ -14129,11 +14086,7 @@
         </is>
       </c>
       <c r="I37" s="7" t="inlineStr"/>
-      <c r="J37" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J37" s="7" t="inlineStr"/>
       <c r="K37" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -14183,7 +14136,7 @@
       </c>
       <c r="V37" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W37" s="7" t="inlineStr">
@@ -14345,11 +14298,7 @@
         </is>
       </c>
       <c r="I39" s="7" t="inlineStr"/>
-      <c r="J39" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J39" s="7" t="inlineStr"/>
       <c r="K39" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -14399,7 +14348,7 @@
       </c>
       <c r="V39" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W39" s="7" t="inlineStr">
@@ -14458,11 +14407,7 @@
         </is>
       </c>
       <c r="I40" s="7" t="inlineStr"/>
-      <c r="J40" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J40" s="7" t="inlineStr"/>
       <c r="K40" s="7" t="inlineStr"/>
       <c r="L40" s="7" t="inlineStr">
         <is>
@@ -14508,7 +14453,7 @@
       </c>
       <c r="V40" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W40" s="7" t="inlineStr">
@@ -14668,7 +14613,7 @@
       <c r="I42" s="7" t="inlineStr"/>
       <c r="J42" s="7" t="inlineStr">
         <is>
-          <t>T7 Course outlines and lesson plans (64 %); T9 Assignments and project descriptions (57 %)</t>
+          <t>T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %); T9 Assignments and project descriptions (57 %)</t>
         </is>
       </c>
       <c r="K42" s="7" t="inlineStr">
@@ -14896,11 +14841,7 @@
         </is>
       </c>
       <c r="I44" s="7" t="inlineStr"/>
-      <c r="J44" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J44" s="7" t="inlineStr"/>
       <c r="K44" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -14954,7 +14895,7 @@
       </c>
       <c r="V44" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W44" s="7" t="inlineStr">
@@ -15015,7 +14956,7 @@
       <c r="I45" s="7" t="inlineStr"/>
       <c r="J45" s="7" t="inlineStr">
         <is>
-          <t>T7 Course outlines and lesson plans (64 %); T5 Personalised learning recommendations (65 %); T11 Questions on regulations and procedures (61 %)</t>
+          <t>T7 Course outlines and lesson plans (64 %); T11 Questions on regulations and procedures (61 %)</t>
         </is>
       </c>
       <c r="K45" s="7" t="inlineStr">
@@ -15132,7 +15073,7 @@
       <c r="I46" s="7" t="inlineStr"/>
       <c r="J46" s="7" t="inlineStr">
         <is>
-          <t>T7 Course outlines and lesson plans (64 %); T5 Personalised learning recommendations (65 %)</t>
+          <t>T7 Course outlines and lesson plans (64 %)</t>
         </is>
       </c>
       <c r="K46" s="7" t="inlineStr">
@@ -16379,11 +16320,7 @@
         </is>
       </c>
       <c r="I57" s="7" t="inlineStr"/>
-      <c r="J57" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J57" s="7" t="inlineStr"/>
       <c r="K57" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -16437,7 +16374,7 @@
       </c>
       <c r="V57" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W57" s="7" t="inlineStr">
@@ -16724,17 +16661,17 @@
       </c>
       <c r="P60" s="7" t="inlineStr">
         <is>
-          <t>Not recommended</t>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="Q60" s="7" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>D25</t>
         </is>
       </c>
       <c r="R60" s="7" t="inlineStr">
         <is>
-          <t>schema:sdLicense; only meaningful once an existing standard is adopted unchanged</t>
+          <t>schema:sdLicense; licence of the structured data, decision deferred (Annex A.7, D25)</t>
         </is>
       </c>
       <c r="S60" s="7" t="inlineStr">
@@ -17025,11 +16962,7 @@
         </is>
       </c>
       <c r="I63" s="7" t="inlineStr"/>
-      <c r="J63" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J63" s="7" t="inlineStr"/>
       <c r="K63" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -17083,7 +17016,7 @@
       </c>
       <c r="V63" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W63" s="7" t="inlineStr">
@@ -17352,7 +17285,7 @@
       <c r="I66" s="7" t="inlineStr"/>
       <c r="J66" s="7" t="inlineStr">
         <is>
-          <t>T3 Solving or explaining problems step by step (87 %); T8 Quiz or exam questions (63 %); T10 Learning objectives and syllabi (52 %)</t>
+          <t>T3 Solving or explaining problems step by step (87 %); T5 Personalised exercise and learning recommendations within a course (65 %); T8 Quiz or exam questions (63 %); T10 Learning objectives and syllabi (52 %)</t>
         </is>
       </c>
       <c r="K66" s="7" t="inlineStr">
@@ -17693,7 +17626,7 @@
       </c>
       <c r="J69" s="7" t="inlineStr">
         <is>
-          <t>T7 Course outlines and lesson plans (64 %); T9 Assignments and project descriptions (57 %)</t>
+          <t>T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %); T9 Assignments and project descriptions (57 %)</t>
         </is>
       </c>
       <c r="K69" s="7" t="inlineStr">
@@ -17804,7 +17737,7 @@
       <c r="I70" s="7" t="inlineStr"/>
       <c r="J70" s="7" t="inlineStr">
         <is>
-          <t>T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised learning recommendations (65 %)</t>
+          <t>T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised exercise and learning recommendations within a course (65 %)</t>
         </is>
       </c>
       <c r="K70" s="7" t="inlineStr">
@@ -18250,11 +18183,7 @@
         </is>
       </c>
       <c r="I74" s="7" t="inlineStr"/>
-      <c r="J74" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J74" s="7" t="inlineStr"/>
       <c r="K74" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -18300,7 +18229,7 @@
       </c>
       <c r="V74" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W74" s="7" t="inlineStr">
@@ -18464,11 +18393,7 @@
         </is>
       </c>
       <c r="I76" s="7" t="inlineStr"/>
-      <c r="J76" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J76" s="7" t="inlineStr"/>
       <c r="K76" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -18518,7 +18443,7 @@
       </c>
       <c r="V76" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W76" s="7" t="inlineStr">
@@ -18575,11 +18500,7 @@
         </is>
       </c>
       <c r="I77" s="7" t="inlineStr"/>
-      <c r="J77" s="7" t="inlineStr">
-        <is>
-          <t>T5 Personalised learning recommendations (65 %)</t>
-        </is>
-      </c>
+      <c r="J77" s="7" t="inlineStr"/>
       <c r="K77" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -18633,7 +18554,7 @@
       </c>
       <c r="V77" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W77" s="7" t="inlineStr">
@@ -19394,4 +19315,1059 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C64"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22.4" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="23.2" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>source code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>reference (APA)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>DOI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>AbuSalih2024</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Abu-Salih, B., &amp; Alotaibi, S. (2024). A systematic literature review of knowledge graph construction and application in education. Heliyon, 10(3), e25383.</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>10.1016/j.heliyon.2024.e25383</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Ali2025</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Ali, A., Collier, A. H., Dewan, U., McDonald, N., &amp; Johri, A. (2025). Analysis of generative AI policies in computing course syllabi. In Proceedings of the 56th ACM Technical Symposium on Computer Science Education V. 1 (pp. 18–24). ACM.</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>10.1145/3641554.3701823</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Alier2025</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Alier, M., Pereira, J., García-Peñalvo, F. J., Casañ, M. J., &amp; Cabré, J. (2025). LAMB: An open-source software framework to create artificial intelligence assistants deployed and integrated into learning management systems. Computer Standards &amp; Interfaces, 92, 103940.</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>10.1016/j.csi.2024.103940</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Bastani2025</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Bastani, H., Bastani, O., Sungu, A., Ge, H., Kabakcı, Ö., &amp; Mariman, R. (2025). Generative AI without guardrails can harm learning: Evidence from high school mathematics. Proceedings of the National Academy of Sciences, 122(26), e2422633122. (Correction: PNAS 122(34), e2518204122 – affiliation of O. Bastani only; findings unaffected.)</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>10.1073/pnas.2422633122</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Bell2009</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Bell, V. (2009). Testing the XCRI-CAP standard on course advertising information at the University of Worcester [Paper]. EUNIS 2009 Congress. University of Worcester Research and Publications. https://eprints.worc.ac.uk/649/</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>BeutlingSpahicBogdanovic2024</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Beutling, N., &amp; Spahic-Bogdanovic, M. (2024). Personalised course recommender: Linking learning objectives and career goals through competencies. Proceedings of the AAAI Symposium Series, 3(1), 72–81. https://doi.org/10.1609/aaaiss.v3i1.31185</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>10.1609/aaaiss.v3i1.31185</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>BruceHillmann2004</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Bruce, T. R., &amp; Hillmann, D. I. (2004). The continuum of metadata quality: Defining, expressing, exploiting. In D. I. Hillmann &amp; E. L. Westbrooks (Eds.), Metadata in practice (pp. 238–256). ALA Editions.</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>CaeiroVelthoven2026</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Caeiro Rodríguez, M., &amp; Velthoven, I. (2026). DACEM policy recommendations (DACEM WP5, D5.5) [Project report]. DACEM Consortium. https://doi.org/10.5281/zenodo.21487970</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>ChandrasekaranMago2022</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Chandrasekaran, D., &amp; Mago, V. (2022). Automating transfer credit assessment: A natural language processing-based approach. Computers, Materials &amp; Continua, 73(2), 2257–2274.</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>10.32604/cmc.2022.027236</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Corbin2025</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Corbin, T., Dawson, P., &amp; Liu, D. (2025). Talk is cheap: Why structural assessment changes are needed for a time of GenAI. Assessment &amp; Evaluation in Higher Education, 50(7), 1087–1097.</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>10.1080/02602938.2025.2503964</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>DACEM2024</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Heidmann, O., Ziogas, D., Lugilde López, A., Marušič, A., Delouis, A., Gomes, B., Vaz de Carvalho, C., Getta, E., Mikic Fonte, F. A., Grosz, G., Todinca, I., Kroubo Dagnini, J., Caeiro Rodríguez, M., Saar, M., Simões, T., Kline, U., &amp; Kozák, V. (2024). Course catalogue mapping (DACEM Activity 2.1) [Project report]. DACEM Consortium. https://doi.org/10.5281/zenodo.14870536</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Daga2016</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Daga, E., d’Aquin, M., Adamou, A., &amp; Brown, S. (2016). The Open University linked data – data.open.ac.uk. Semantic Web, 7(2), 183–191.</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>10.3233/SW-150182</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Dietze2017</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Dietze, S., Taibi, D., Yu, R., Barker, P., &amp; d’Aquin, M. (2017). Analysing and improving embedded markup of learning resources on the web. In Proceedings of the 26th International Conference on World Wide Web Companion (pp. 283–292). IW3C2/ACM.</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>10.1145/3041021.3054160</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Doughty2024</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Doughty, J., Wan, Z., Bompelli, A., Qayum, J., Wang, T., Zhang, J., Zheng, Y., Doyle, A., Sridhar, P., Agarwal, A., Bogart, C., Keylor, E., Kultur, C., Savelka, J., &amp; Sakr, M. (2024). A comparative study of AI-generated (GPT-4) and human-crafted MCQs in programming education. In Proceedings of the 26th Australasian Computing Education Conference (ACE 2024) (pp. 114–123). ACM. https://doi.org/10.1145/3636243.3636256</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>10.1145/3636243.3636256</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Duarte2024</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Duarte, R., Lacerda Nobre, Â., Pimentel, F., &amp; Jacquinet, M. (2024). Broader terms curriculum mapping: Using natural language processing and visual-supported communication to create representative program planning experiences. Applied System Innovation, 7(1), 7.</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>10.3390/asi7010007</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Eastwood2026</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Eastwood, M., Narne, H., Hilby, J., Denny, P., Aggarwal, A., &amp; Kapoor, A. (2026). Guardrails or roadblocks? Effects of pedagogical style and context awareness in AI teaching assistants for programming [Preprint]. arXiv. https://doi.org/10.48550/arXiv.2609.29995</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>10.48550/arXiv.2609.29995</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>EC_ELM_ontology</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>European Commission. (n.d.). Europass Learning Model ontology (Revision 3.2.0). Retrieved October 18, 2026, from https://europa.eu/europass/elm-browser/documentation/rdf/ontology/documentation/elm.html</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>EUF2026_OCCAPI</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>European University Foundation. (2026). Open Course Catalogue API (OCCAPI) (Version 2.0.0-beta2) [API specification, draft]. https://occapi.uni-foundation.eu/specification/v2</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Ferrell2013</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Ferrell, G., &amp; Hillicks, J. (2013). Opening Pandora's box: Implementing a standards-based approach to the management of course information in UK higher education. In EUNIS 2013 Congress Proceedings. Riga Technical University.</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>10.7250/eunis.2013.031</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Groher2026</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Groher, I., Heissenberger, P., &amp; Vierhauser, M. (2026). Design and deployment of a course-aware AI tutor in an introductory programming course [Preprint, accepted at the 18th International Conference on Computer Supported Education (CSEDU 2026)]. arXiv. https://doi.org/10.48550/arXiv.2604.11836</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>10.48550/arXiv.2604.11836</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Harrington2023</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Harrington, C. (2023). Is the syllabus passé? Student and faculty perceptions. Journal of the Scholarship of Teaching and Learning, 23(4), 19–32.</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>10.14434/josotl.v23i4.34371</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Heil2024</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Heil, A., Olaniran, A., Gormally, C., &amp; Brickman, P. (2024). It’s in the syllabus: What syllabi tell us about introductory biology courses. CBE—Life Sciences Education, 23(3), ar37.</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>10.1187/cbe.23-05-0081</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Heppner2019</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Heppner, A., Pawar, A., Kivi, D., &amp; Mago, V. (2019). Automating articulation: Applying natural language processing to post-secondary credit transfer. IEEE Access, 7, 48295–48306. https://doi.org/10.1109/ACCESS.2019.2910145</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>10.1109/ACCESS.2019.2910145</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>HillmannPhipps2007</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Hillmann, D. I., &amp; Phipps, J. (2007). Application profiles: Exposing and enforcing metadata quality. In Proceedings of the International Conference on Dublin Core and Metadata Applications (DC-2007) (pp. 52–62). Dublin Core Metadata Initiative.</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>10.23106/dcmi.952108665</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>HoLam2026</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Ho, T.-L., &amp; Lam, T.-P. (2026). EduMSRA: A multi-source educational research agent integrating retrieval-augmented generation and Model Context Protocol for adaptive intelligent tutoring systems. Applied Sciences, 16(9), 4400.</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>10.3390/app16094400</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Hou2026</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Hou, I., Xiong, Z., Guo, P. J., &amp; Wang, A. Y. (2026). “Bespoke bots”: Diverse instructor needs for customizing generative AI classroom chatbots. In Proceedings of the 2026 CHI Conference on Human Factors in Computing Systems (CHI '26) (Article 705, pp. 1–10). ACM. https://doi.org/10.1145/3772318.3791491</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>10.1145/3772318.3791491</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>Huerta2023</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Huerta, E. A., Blaiszik, B., Brinson, L. C., Bouchard, K. E., Diaz, D., Doglioni, C., … Zhu, R. (2023). FAIR for AI: An interdisciplinary and international community building perspective. Scientific Data, 10, 487.</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>10.1038/s41597-023-02298-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Humble2025</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Humble, N. (2025). Higher education AI policies—A document analysis of university guidelines. European Journal of Education, 60(3), e70214.</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>10.1111/ejed.70214</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>IEEE2025_2881</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>IEEE. (2025). IEEE standard for learning metadata terms (IEEE Std 2881-2025). https://doi.org/10.1109/IEEESTD.2025.11192251</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Jensen2024</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Jensen, C. G., Dau, S., &amp; Gade, P. (2024). The role of AI chatbots in scaffolding: Linking learning outcomes with assessment. Learning Tech – Tidsskrift for læremidler, didaktik og teknologi, (14), 73–97. https://doi.org/10.7146/lt.v9i14.141213</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>10.7146/lt.v9i14.141213</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Kazemitabaar2024</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Kazemitabaar, M., Ye, R., Wang, X., Henley, A. Z., Denny, P., Craig, M., &amp; Grossman, T. (2024). CodeAid: Evaluating a classroom deployment of an LLM-based programming assistant that balances student and educator needs. In Proceedings of the CHI Conference on Human Factors in Computing Systems (CHI '24) (pp. 1–20). ACM. https://doi.org/10.1145/3613904.3642773</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>10.1145/3613904.3642773</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Kestin2025</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Kestin, G., Miller, K., Klales, A., Milbourne, T., &amp; Ponti, G. (2025). AI tutoring outperforms in-class active learning: An RCT introducing a novel research-based design in an authentic educational setting. Scientific Reports, 15, 17458.</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>10.1038/s41598-025-97652-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>KIM2023_AMB</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Kompetenzzentrum Interoperable Metadaten. (2023). Allgemeines Metadatenprofil für Bildungsressourcen (AMB) (Version 2023-10-19). https://w3id.org/kim/amb/20231019/</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Kolagar2025</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Kolagar, Z., Zalkow, F., &amp; Zarcone, A. (2025). Investigating methods for mapping learning objectives to Bloom’s revised taxonomy in course descriptions for higher education. In Proceedings of the 20th Workshop on Innovative Use of NLP for Building Educational Applications (BEA 2025) (pp. 415–445). Association for Computational Linguistics. https://doi.org/10.18653/v1/2025.bea-1.32</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>10.18653/v1/2025.bea-1.32</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Li2022</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Li, Y., Raković, M., Poh, B. X., Gašević, D., &amp; Chen, G. (2022). Automatic classification of learning objectives based on Bloom’s taxonomy. In A. Mitrovic &amp; N. Bosch (Eds.), Proceedings of the 15th International Conference on Educational Data Mining (pp. 530–537). International Educational Data Mining Society. https://doi.org/10.5281/zenodo.6853191</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>10.5281/zenodo.6853191</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Liffiton2023</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Liffiton, M., Sheese, B. E., Savelka, J., &amp; Denny, P. (2023). CodeHelp: Using large language models with guardrails for scalable support in programming classes. In Proceedings of the 23rd Koli Calling International Conference on Computing Education Research (pp. 1–11). ACM. https://doi.org/10.1145/3631802.3631830</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>10.1145/3631802.3631830</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>Liu2024CS50</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Liu, R., Zenke, C., Liu, C., Holmes, A., Thornton, P., &amp; Malan, D. J. (2024). Teaching CS50 with AI: Leveraging generative artificial intelligence in computer science education. In Proceedings of the 55th ACM Technical Symposium on Computer Science Education V. 1 (pp. 750–756). ACM.</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>10.1145/3626252.3630938</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>Luo2024</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Luo, J. (2024). A critical review of GenAI policies in higher education assessment: A call to reconsider the "originality" of students' work. Assessment &amp; Evaluation in Higher Education, 49(5), 651–664.</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>10.1080/02602938.2024.2309963</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>McDonald2025</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>McDonald, N., Johri, A., Ali, A., &amp; Collier, A. H. (2025). Generative artificial intelligence in higher education: Evidence from an analysis of institutional policies and guidelines. Computers in Human Behavior: Artificial Humans, 3, 100121. https://doi.org/10.1016/j.chbah.2025.100121</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>10.1016/j.chbah.2025.100121</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>Menzel2023</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Menzel, M. (2023). Developing a metadata profile for higher education OER repositories. In D. Otto, G. Scharnberg, M. Kerres, &amp; O. Zawacki-Richter (Eds.), Distributed learning ecosystems: Concepts, resources, and repositories (pp. 263–278). Springer VS. https://doi.org/10.1007/978-3-658-38703-7_14</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>MusgraveSumner2026</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Musgrave, S., &amp; Sumner, J. L. (2026). Using AI to assess demographic balance of syllabi and bibliographies. PS: Political Science &amp; Politics, 59(4), 722–730. https://doi.org/10.1017/S104909652610198X</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>10.1017/S104909652610198X</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>Nahhas2019</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Nahhas, S., Bamasag, O. O., &amp; Khemakhem, M. (2019). Bridging education and labor skills by a novel competency-based course linked-data model. IEEE Access, 7, 119087–119098.</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>10.1109/ACCESS.2019.2937233</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>OellersRoertgen2024</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Oellers, M., &amp; Rörtgen, S. (2024). Kompendium: Didaktische Metadaten (Version 1.0.2). Zenodo. https://doi.org/10.5281/zenodo.10828758</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>Otto2023</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Otto, D., Scharnberg, G., Kerres, M., &amp; Zawacki-Richter, O. (Eds.). (2023). Distributed learning ecosystems: Concepts, resources, and repositories. Springer VS. https://doi.org/10.1007/978-3-658-38703-7</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>Palmer2014</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Palmer, M. S., Bach, D. J., &amp; Streifer, A. C. (2014). Measuring the promise: A learning-focused syllabus rubric. To Improve the Academy, 33(1), 14–36.</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>10.1002/tia2.20004</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>PardosNam2020</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Pardos, Z. A., &amp; Nam, A. J. H. (2020). A university map of course knowledge. PLOS ONE, 15(9), e0233207. https://doi.org/10.1371/journal.pone.0233207</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>10.1371/journal.pone.0233207</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>Pereira2024</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Pereira, E., Nsair, S., Pereira, L. R., &amp; Grant, K. (2024). Constructive alignment in a graduate-level project management course: An innovative framework using large language models. International Journal of Educational Technology in Higher Education, 21, 25.</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>10.1186/s41239-024-00457-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>Perkins2024</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Perkins, M., Furze, L., Roe, J., &amp; MacVaugh, J. (2024). The Artificial Intelligence Assessment Scale (AIAS): A framework for ethical integration of generative AI in educational assessment. Journal of University Teaching and Learning Practice, 21(6). https://doi.org/10.53761/q3azde36</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>10.53761/q3azde36</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>Perkins2025</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Perkins, M., Roe, J., &amp; Furze, L. (2025). Reimagining the Artificial Intelligence Assessment Scale (AIAS): A refined framework for educational assessment. Journal of University Teaching and Learning Practice, 22(7). https://doi.org/10.53761/rrm4y757</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>10.53761/rrm4y757</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>Riahi2026</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Riahi, B., Ozturk, D., Guth, A., Li, J., Singh, D. P., Tian, X., Chiu, J., Lytle, N., Barnes, T., &amp; Cateté, V. (2026). Will it teach as intended? How teachers configure educational AI chatbots [Preprint]. arXiv. https://doi.org/10.48550/arXiv.2609.29993</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>10.48550/arXiv.2609.29993</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>Sajja2023</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Sajja, R., Sermet, Y., Cwiertny, D., &amp; Demir, I. (2023). Platform-independent and curriculum-oriented intelligent assistant for higher education. International Journal of Educational Technology in Higher Education, 20, 42. https://doi.org/10.1186/s41239-023-00412-7</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>10.1186/s41239-023-00412-7</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>SchemaOrg2026</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Schema.org. (2026). Course, CourseInstance, Syllabus. Retrieved October 18, 2026, from https://schema.org/Course</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>Shaikh2021</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Shaikh, S., Daudpotta, S. M., &amp; Imran, A. S. (2021). Bloom's learning outcomes' automatic classification using LSTM and pretrained word embeddings. IEEE Access, 9, 117887–117909.</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>10.1109/ACCESS.2021.3106443</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>SimoesTueck2025</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Simões, T., &amp; Tück, C. (2025). Development of technical standards to support sharing of quality and course information: Technical specifications (J. Ehrenreich, Ed.; QualityLink report on Work Package 3). QualityLink. https://quality-link.eu/wp-content/uploads/sites/90/2026/08/QualityLink_WP3_Full_Report_Technical_Standards.pdf</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>Stanny2016</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Stanny, C. J. (2016). Reevaluating Bloom’s taxonomy: What measurable verbs can and cannot say about student learning. Education Sciences, 6(4), 37. https://doi.org/10.3390/educsci6040037</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>10.3390/educsci6040037</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>Szasz2017</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Szász, B., Fleiner, R., &amp; Micsik, A. (2017). A case study on linked data for university courses. In I. Ciuciu et al. (Eds.), On the move to meaningful internet systems: OTM 2016 workshops (LNCS 10034, pp. 265–276). Springer.</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>10.1007/978-3-319-55961-2_27</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>Taneja2024</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Taneja, K., Maiti, P., Kakar, S., Guruprasad, P., Rao, S., &amp; Goel, A. K. (2024). Jill Watson: A virtual teaching assistant powered by ChatGPT. In Artificial Intelligence in Education (AIED 2024) (pp. 324–337). Springer. https://doi.org/10.1007/978-3-031-64302-6_23 (preprint: arXiv:2405.11070)</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>10.1007/978-3-031-64302-6_23</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>Tani2013</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Tani, A., Candela, L., &amp; Castelli, D. (2013). Dealing with metadata quality: The legacy of digital library efforts. Information Processing &amp; Management, 49(6), 1194–1205.</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>10.1016/j.ipm.2013.05.003</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>TapiaLeon2018</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Tapia-León, M., Carrera Rivera, A., Chicaiza, J., &amp; Luján-Mora, S. (2018). The use of ontologies for syllabus representation. In 2018 17th International Conference on Information Technology Based Higher Education and Training (ITHET) (pp. 1–7). IEEE.</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>10.1109/ITHET.2018.8424788</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>Verbeken2026</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Verbeken, B., Van den Broeck, J., De Cleyn, I., Engels, N., Algaba, A., Van Luchene, S., &amp; Ginis, V. (2026). Scalable classification of course information sheets using large language models: A reusable institutional method for academic quality assurance (arXiv:2603.13562) [Preprint]. arXiv.</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>10.48550/arXiv.2603.13562</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>Weaver2024</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Weaver, K. D. (2024). The Artificial Intelligence Disclosure (AID) Framework: An introduction. College &amp; Research Libraries News, 85(10), 407–411.</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>10.5860/crln.85.10.407</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>Wilkinson2016</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Wilkinson, M. D., Dumontier, M., Aalbersberg, I. J., Appleton, G., Axton, M., Baak, A., … Mons, B. (2016). The FAIR guiding principles for scientific data management and stewardship. Scientific Data, 3, 160018.</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>10.1038/sdata.2016.18</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>Zaki2023</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>Zaki, N., Turaev, S., Shuaib, K., Krishnan, A., &amp; Mohamed, E. A. (2023). Automating the mapping of course learning outcomes to program learning outcomes using natural language processing for accurate educational program evaluation. Education and Information Technologies, 28(12), 16723–16742.</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>10.1007/s10639-023-11877-4</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update AI-use evidence in profile.xlsx after review of the WP2 matrix
Use lists per element (Elements: evidence) and per candidate field
(Candidate fields: p3_wp2, m_p3_use) follow the reviewed derivation
matrix. Definitions, mappings, tiers, schema and shapes are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -755,7 +755,7 @@
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓5 · P2 6/10; WP4 Md 4, 73 %, ✘ · P3 T11</t>
+          <t>P1 ✓5 · P2 6/10; WP4 Md 4, 73 %, ✘ · P3 –</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 0/10; WP4 Md 5, 82 %, ✔ · P3 A3, A4</t>
+          <t>P1 ✓3 · P2 0/10; WP4 Md 5, 82 %, ✔ · P3 T11, A3, A4</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
@@ -1240,7 +1240,7 @@
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓5 · P2 10/10; WP4 Md 5, 100 %, ✔ · P3 T1, T2, T5, T7; MyAI University</t>
+          <t>P1 ✓5 · P2 10/10; WP4 Md 5, 100 %, ✔ · P3 T1, T2, T5, T7, T10; MyAI University</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 6/10 (+3); WP4 Md 4, 100 %, ✔ · P3 T1, T2, T5, T7, T8</t>
+          <t>P1 ✓2 · P2 6/10 (+3); WP4 Md 4, 100 %, ✔ · P3 T1, T2, T3, T4, T5, T7, T8, T9, T10</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓4 · P2 4/10 (+4); WP4 Md 4, 70 %, ✘ · P3 T1, T2, T5, T10; MyAI University</t>
+          <t>P1 ✓4 · P2 4/10 (+4); WP4 Md 4, 70 %, ✘ · P3 T1, T2, T5, T7, T8, T10; MyAI University</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 10/10; manual course-specific ●6/10; WP4 Md 5, 90 %, ✔ · P3 T2, T3, T4, T5, T7, T8, T10; design input, MyAI University</t>
+          <t>P1 ✓3 · P2 10/10; manual course-specific ●6/10; WP4 Md 5, 90 %, ✔ · P3 T2, T3, T4, T5, T7, T8, T9, T10, T12; design input, MyAI University</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 9/10; WP4 Md 4, 90 %, ✔ · P3 T7; MyAI University</t>
+          <t>P1 ✓3 · P2 9/10; WP4 Md 4, 90 %, ✔ · P3 T7, T9, T10; MyAI University</t>
         </is>
       </c>
       <c r="S14" s="2" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓4 · P2 9/10 (+1); WP4 Md 4, 80 %, ✔ · P3 T5, T7, T9; MyAI University</t>
+          <t>P1 ✓4 · P2 9/10 (+1); WP4 Md 4, 80 %, ✔ · P3 T5, T7, T9, T10; MyAI University</t>
         </is>
       </c>
       <c r="S16" s="2" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓1 · P2 10/10; manual methods + weights ●4/10; WP4 Md 4, 80 %, ✔ · P3 T4, T8, T9, T11; MyAI University</t>
+          <t>P1 ✓1 · P2 10/10; manual methods + weights ●4/10; WP4 Md 4, 80 %, ✔ · P3 T4, T7, T8, T9, T10, T11, T12; MyAI University</t>
         </is>
       </c>
       <c r="S17" s="2" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓2 (scale) / ✗ (graded vs pass/fail) · P2 8/10 (+2); WP4 Md 4, 80 %, ✔ · P3 T4, T11</t>
+          <t>P1 ✓2 (scale) / ✗ (graded vs pass/fail) · P2 8/10 (+2); WP4 Md 4, 80 %, ✔ · P3 T4, T11, T12</t>
         </is>
       </c>
       <c r="S18" s="2" t="inlineStr">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓4 · P2 8/10; WP4 Md 4, 82 %, ✔ · P3 T1, A4</t>
+          <t>P1 ✓4 · P2 8/10; WP4 Md 4, 82 %, ✔ · P3 T1, T2, T3, T4, T5, T6, T8, A3, A4</t>
         </is>
       </c>
       <c r="S19" s="2" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
-          <t>P1 hook · P2 0/10 (no Bloom tagging in any document) · P3 T3, T5, T8, T10; design input, MyAI University</t>
+          <t>P1 hook · P2 0/10 (no Bloom tagging in any document) · P3 T2, T3, T4, T5, T7, T8, T9, T10, T12; design input, MyAI University</t>
         </is>
       </c>
       <c r="S20" s="3" t="inlineStr">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="R23" s="3" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 competences assessed 1/10 (+3); manual ●2/10; WP4 Md 5, 80 %, ✔ · P3 T4, T5, T8, T12; WP4: structured outcome–assessment mapping for most courses 3/11, for some 2/11; design input</t>
+          <t>P1 ✓2 · P2 competences assessed 1/10 (+3); manual ●2/10; WP4 Md 5, 80 %, ✔ · P3 T4, T7, T8, T9, T12; WP4: structured outcome–assessment mapping for most courses 3/11, for some 2/11; design input</t>
         </is>
       </c>
       <c r="S23" s="3" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="R25" s="3" t="inlineStr">
         <is>
-          <t>P1 ✓1 · P2 2/10; WP4 Md 4, 70 %, ✘ · P3 T4, T12</t>
+          <t>P1 ✓1 · P2 2/10; WP4 Md 4, 70 %, ✘ · P3 T4, T8, T9, T10, T12</t>
         </is>
       </c>
       <c r="S25" s="3" t="inlineStr">
@@ -3180,7 +3180,7 @@
       </c>
       <c r="R27" s="3" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 0/10 (+4 in text); WP4 Md 4, 91 %, ✔ · P3 T2, T5; MyAI University</t>
+          <t>P1 ✓3 · P2 0/10 (+4 in text); WP4 Md 4, 91 %, ✔ · P3 T2, T5, T7, T10; MyAI University</t>
         </is>
       </c>
       <c r="S27" s="3" t="inlineStr">
@@ -3277,7 +3277,7 @@
       </c>
       <c r="R28" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 n.m. (no field in any partner document) · P3 T2, T3; design input</t>
+          <t>P1 ✗ · P2 n.m. (no field in any partner document) · P3 T2, T3, T5, T8; design input</t>
         </is>
       </c>
       <c r="S28" s="3" t="inlineStr">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="R29" s="3" t="inlineStr">
         <is>
-          <t>P1 hook · P2 2/10 (+2); WP4 Md 4, 80 %, ✔ · P3 T2, T5; MyAI University</t>
+          <t>P1 hook · P2 2/10 (+2); WP4 Md 4, 80 %, ✔ · P3 T2, T3, T5, T7, T10; MyAI University</t>
         </is>
       </c>
       <c r="S29" s="3" t="inlineStr">
@@ -3471,7 +3471,7 @@
       </c>
       <c r="R30" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 no field in any partner; AI rules found only at assessment level (A12) · P3 T3, A1; all reported institutional policies PDF/web only; design input</t>
+          <t>P1 ✗ · P2 no field in any partner; AI rules found only at assessment level (A12) · P3 T3, T11, A1, A2; all reported institutional policies PDF/web only; design input</t>
         </is>
       </c>
       <c r="S30" s="3" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="R31" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 1/10 (permitted aids of individual exams, 7 of 125 module descriptions) · P3 T9, A1, A2; institutional policies cover assessments at 7 of 9; design input</t>
+          <t>P1 ✗ · P2 1/10 (permitted aids of individual exams, 7 of 125 module descriptions) · P3 T3, T4, T8, T9, T11, A1, A2; institutional policies cover assessments at 7 of 9; design input</t>
         </is>
       </c>
       <c r="S31" s="3" t="inlineStr">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="R33" s="3" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 0/10; WP4 Md 4, 64 %, ✘ · P3 A4; MyAI University</t>
+          <t>P1 ✓3 · P2 0/10; WP4 Md 4, 64 %, ✘ · P3 MyAI University</t>
         </is>
       </c>
       <c r="S33" s="3" t="inlineStr">
@@ -4344,7 +4344,7 @@
       </c>
       <c r="R39" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓3 (but conflated with cycle) · P2 1/10 (+3); WP4 Md 4, 60 %, ✘ · P3 T2, T5; MyAI University</t>
+          <t>P1 ✓3 (but conflated with cycle) · P2 1/10 (+3); WP4 Md 4, 60 %, ✘ · P3 T1, T2, T5; MyAI University</t>
         </is>
       </c>
       <c r="S39" s="4" t="inlineStr">
@@ -4441,7 +4441,7 @@
       </c>
       <c r="R40" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 0/10; WP4 Md 4, 60 %, ✘ · P3 T10; MyAI University</t>
+          <t>P1 ✓3 · P2 0/10; WP4 Md 4, 60 %, ✘ · P3 MyAI University</t>
         </is>
       </c>
       <c r="S40" s="4" t="inlineStr">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="R48" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 coordinator 6/10; WP4 Md 4, 55 %, ✘ · P3 T11</t>
+          <t>P1 ✓3 · P2 coordinator 6/10; WP4 Md 4, 55 %, ✘ · P3 –</t>
         </is>
       </c>
       <c r="S48" s="4" t="inlineStr">
@@ -7157,7 +7157,7 @@
       </c>
       <c r="R68" s="5" t="inlineStr">
         <is>
-          <t>P1 ✓5 (date group) · P2 currency 2/10 (+2); WP4 Md 4, 64 %, ✘ · P3 A3; MyAI University</t>
+          <t>P1 ✓5 (date group) · P2 currency 2/10 (+2); WP4 Md 4, 64 %, ✘ · P3 T11, A3; MyAI University</t>
         </is>
       </c>
       <c r="S68" s="5" t="inlineStr">
@@ -7448,7 +7448,7 @@
       </c>
       <c r="R71" s="5" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 n.m.; WP4 Md 4, 64 %, ✘ · P3 A3; MyAI University</t>
+          <t>P1 ✓2 · P2 n.m.; WP4 Md 4, 64 %, ✘ · P3 T11, A3; MyAI University</t>
         </is>
       </c>
       <c r="S71" s="5" t="inlineStr">
@@ -8224,7 +8224,7 @@
       </c>
       <c r="R79" s="5" t="inlineStr">
         <is>
-          <t>P1 ✓1 (schema.org) · P2 bilingual versions at 2/10 (manual review) · P3 T6</t>
+          <t>P1 ✓1 (schema.org) · P2 bilingual versions at 2/10 (manual review) · P3 –</t>
         </is>
       </c>
       <c r="S79" s="5" t="inlineStr">
@@ -10135,11 +10135,7 @@
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr"/>
-      <c r="J2" s="7" t="inlineStr">
-        <is>
-          <t>T11 Questions on regulations and procedures (61 %)</t>
-        </is>
-      </c>
+      <c r="J2" s="7" t="inlineStr"/>
       <c r="K2" s="7" t="inlineStr"/>
       <c r="L2" s="7" t="inlineStr">
         <is>
@@ -10193,7 +10189,7 @@
       </c>
       <c r="V2" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W2" s="7" t="inlineStr">
@@ -10581,7 +10577,7 @@
       <c r="I6" s="7" t="inlineStr"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>A3 More trust in AI output with visible sources (67 %); A4 Course-specific documents given to AI tools by hand (42 %)</t>
+          <t>T11 Questions on regulations and procedures (61 %); A3 More trust in AI output with visible sources (67 %); A4 Course-specific documents given to AI tools by hand (42 %)</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr"/>
@@ -11679,11 +11675,7 @@
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr"/>
-      <c r="J16" s="7" t="inlineStr">
-        <is>
-          <t>T11 Questions on regulations and procedures (61 %)</t>
-        </is>
-      </c>
+      <c r="J16" s="7" t="inlineStr"/>
       <c r="K16" s="7" t="inlineStr"/>
       <c r="L16" s="7" t="inlineStr">
         <is>
@@ -11733,7 +11725,7 @@
       </c>
       <c r="V16" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W16" s="7" t="inlineStr">
@@ -11794,7 +11786,7 @@
       <c r="I17" s="7" t="inlineStr"/>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised exercise and learning recommendations within a course (65 %)</t>
+          <t>T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %); T10 Learning objectives and syllabi (52 %)</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -11911,7 +11903,7 @@
       <c r="I18" s="7" t="inlineStr"/>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %)</t>
+          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %); T10 Learning objectives and syllabi (52 %)</t>
         </is>
       </c>
       <c r="K18" s="7" t="inlineStr">
@@ -12141,7 +12133,7 @@
       <c r="I20" s="7" t="inlineStr"/>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %); T8 Quiz or exam questions (63 %)</t>
+          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T3 Solving or explaining problems step by step (87 %); T4 Exam preparation (86 %); T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %); T8 Quiz or exam questions (63 %); T9 Assignments and project descriptions (57 %); T10 Learning objectives and syllabi (52 %)</t>
         </is>
       </c>
       <c r="K20" s="7" t="inlineStr"/>
@@ -12597,7 +12589,7 @@
       <c r="I24" s="7" t="inlineStr"/>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>T1 Summarising or simplifying reading material (92 %); A4 Course-specific documents given to AI tools by hand (42 %)</t>
+          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T3 Solving or explaining problems step by step (87 %); T4 Exam preparation (86 %); T5 Personalised exercise and learning recommendations within a course (65 %); T6 Language learning or translation support (78 %); T8 Quiz or exam questions (63 %); A3 More trust in AI output with visible sources (67 %); A4 Course-specific documents given to AI tools by hand (42 %)</t>
         </is>
       </c>
       <c r="K24" s="7" t="inlineStr"/>
@@ -12938,11 +12930,7 @@
           <t>Licence information requested</t>
         </is>
       </c>
-      <c r="J27" s="7" t="inlineStr">
-        <is>
-          <t>A4 Course-specific documents given to AI tools by hand (42 %)</t>
-        </is>
-      </c>
+      <c r="J27" s="7" t="inlineStr"/>
       <c r="K27" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -12992,7 +12980,7 @@
       </c>
       <c r="V27" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W27" s="7" t="inlineStr">
@@ -13164,7 +13152,7 @@
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>T2 Explanations of concepts (AI as tutor) (88 %); T3 Solving or explaining problems step by step (87 %); T4 Exam preparation (86 %); T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %); T8 Quiz or exam questions (63 %); T10 Learning objectives and syllabi (52 %)</t>
+          <t>T2 Explanations of concepts (AI as tutor) (88 %); T3 Solving or explaining problems step by step (87 %); T4 Exam preparation (86 %); T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %); T8 Quiz or exam questions (63 %); T9 Assignments and project descriptions (57 %); T10 Learning objectives and syllabi (52 %); T12 Written feedback and grading rubrics (26 %)</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
@@ -13285,7 +13273,7 @@
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>T4 Exam preparation (86 %); T5 Personalised exercise and learning recommendations within a course (65 %); T8 Quiz or exam questions (63 %); T12 Written feedback and grading rubrics (26 %)</t>
+          <t>T4 Exam preparation (86 %); T7 Course outlines and lesson plans (64 %); T8 Quiz or exam questions (63 %); T9 Assignments and project descriptions (57 %); T12 Written feedback and grading rubrics (26 %)</t>
         </is>
       </c>
       <c r="K30" s="7" t="inlineStr">
@@ -13400,11 +13388,7 @@
         </is>
       </c>
       <c r="I31" s="7" t="inlineStr"/>
-      <c r="J31" s="7" t="inlineStr">
-        <is>
-          <t>T10 Learning objectives and syllabi (52 %)</t>
-        </is>
-      </c>
+      <c r="J31" s="7" t="inlineStr"/>
       <c r="K31" s="7" t="inlineStr">
         <is>
           <t>MyAI University</t>
@@ -13458,7 +13442,7 @@
       </c>
       <c r="V31" s="7" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W31" s="7" t="inlineStr">
@@ -13519,7 +13503,7 @@
       <c r="I32" s="7" t="inlineStr"/>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T10 Learning objectives and syllabi (52 %); T5 Personalised exercise and learning recommendations within a course (65 %)</t>
+          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %); T8 Quiz or exam questions (63 %); T10 Learning objectives and syllabi (52 %)</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
@@ -13632,7 +13616,7 @@
       <c r="I33" s="7" t="inlineStr"/>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised exercise and learning recommendations within a course (65 %)</t>
+          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised exercise and learning recommendations within a course (65 %)</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
@@ -13971,7 +13955,7 @@
       <c r="I36" s="7" t="inlineStr"/>
       <c r="J36" s="7" t="inlineStr">
         <is>
-          <t>T2 Explanations of concepts (AI as tutor) (88 %); T5 Personalised exercise and learning recommendations within a course (65 %)</t>
+          <t>T2 Explanations of concepts (AI as tutor) (88 %); T3 Solving or explaining problems step by step (87 %); T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %); T10 Learning objectives and syllabi (52 %)</t>
         </is>
       </c>
       <c r="K36" s="7" t="inlineStr">
@@ -14613,7 +14597,7 @@
       <c r="I42" s="7" t="inlineStr"/>
       <c r="J42" s="7" t="inlineStr">
         <is>
-          <t>T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %); T9 Assignments and project descriptions (57 %)</t>
+          <t>T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %); T9 Assignments and project descriptions (57 %); T10 Learning objectives and syllabi (52 %)</t>
         </is>
       </c>
       <c r="K42" s="7" t="inlineStr">
@@ -15073,7 +15057,7 @@
       <c r="I46" s="7" t="inlineStr"/>
       <c r="J46" s="7" t="inlineStr">
         <is>
-          <t>T7 Course outlines and lesson plans (64 %)</t>
+          <t>T7 Course outlines and lesson plans (64 %); T9 Assignments and project descriptions (57 %); T10 Learning objectives and syllabi (52 %)</t>
         </is>
       </c>
       <c r="K46" s="7" t="inlineStr">
@@ -15303,7 +15287,7 @@
       <c r="I48" s="7" t="inlineStr"/>
       <c r="J48" s="7" t="inlineStr">
         <is>
-          <t>T4 Exam preparation (86 %); T8 Quiz or exam questions (63 %); T9 Assignments and project descriptions (57 %); T11 Questions on regulations and procedures (61 %)</t>
+          <t>T4 Exam preparation (86 %); T7 Course outlines and lesson plans (64 %); T8 Quiz or exam questions (63 %); T9 Assignments and project descriptions (57 %); T10 Learning objectives and syllabi (52 %); T11 Questions on regulations and procedures (61 %); T12 Written feedback and grading rubrics (26 %)</t>
         </is>
       </c>
       <c r="K48" s="7" t="inlineStr">
@@ -15420,7 +15404,7 @@
       <c r="I49" s="7" t="inlineStr"/>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>T4 Exam preparation (86 %); T12 Written feedback and grading rubrics (26 %)</t>
+          <t>T4 Exam preparation (86 %); T8 Quiz or exam questions (63 %); T9 Assignments and project descriptions (57 %); T10 Learning objectives and syllabi (52 %); T12 Written feedback and grading rubrics (26 %)</t>
         </is>
       </c>
       <c r="K49" s="7" t="inlineStr"/>
@@ -15533,7 +15517,7 @@
       <c r="I50" s="7" t="inlineStr"/>
       <c r="J50" s="7" t="inlineStr">
         <is>
-          <t>T4 Exam preparation (86 %); T11 Questions on regulations and procedures (61 %)</t>
+          <t>T4 Exam preparation (86 %); T11 Questions on regulations and procedures (61 %); T12 Written feedback and grading rubrics (26 %)</t>
         </is>
       </c>
       <c r="K50" s="7" t="inlineStr"/>
@@ -15753,11 +15737,7 @@
         </is>
       </c>
       <c r="I52" s="7" t="inlineStr"/>
-      <c r="J52" s="7" t="inlineStr">
-        <is>
-          <t>T6 Language learning or translation support (78 %)</t>
-        </is>
-      </c>
+      <c r="J52" s="7" t="inlineStr"/>
       <c r="K52" s="7" t="inlineStr"/>
       <c r="L52" s="7" t="inlineStr">
         <is>
@@ -15807,7 +15787,7 @@
       </c>
       <c r="V52" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="W52" s="7" t="inlineStr">
@@ -17285,7 +17265,7 @@
       <c r="I66" s="7" t="inlineStr"/>
       <c r="J66" s="7" t="inlineStr">
         <is>
-          <t>T3 Solving or explaining problems step by step (87 %); T5 Personalised exercise and learning recommendations within a course (65 %); T8 Quiz or exam questions (63 %); T10 Learning objectives and syllabi (52 %)</t>
+          <t>T2 Explanations of concepts (AI as tutor) (88 %); T3 Solving or explaining problems step by step (87 %); T4 Exam preparation (86 %); T5 Personalised exercise and learning recommendations within a course (65 %); T7 Course outlines and lesson plans (64 %); T8 Quiz or exam questions (63 %); T9 Assignments and project descriptions (57 %); T10 Learning objectives and syllabi (52 %); T12 Written feedback and grading rubrics (26 %)</t>
         </is>
       </c>
       <c r="K66" s="7" t="inlineStr">
@@ -17852,7 +17832,7 @@
       <c r="I71" s="7" t="inlineStr"/>
       <c r="J71" s="7" t="inlineStr">
         <is>
-          <t>T2 Explanations of concepts (AI as tutor) (88 %); T3 Solving or explaining problems step by step (87 %)</t>
+          <t>T2 Explanations of concepts (AI as tutor) (88 %); T3 Solving or explaining problems step by step (87 %); T5 Personalised exercise and learning recommendations within a course (65 %); T8 Quiz or exam questions (63 %)</t>
         </is>
       </c>
       <c r="K71" s="7" t="inlineStr">
@@ -17963,7 +17943,7 @@
       <c r="I72" s="7" t="inlineStr"/>
       <c r="J72" s="7" t="inlineStr">
         <is>
-          <t>A1 Clear rules for AI use in assessed work (79 %); T3 Solving or explaining problems step by step (87 %)</t>
+          <t>T3 Solving or explaining problems step by step (87 %); T11 Questions on regulations and procedures (61 %); A1 Clear rules for AI use in assessed work (79 %); A2 Students should always disclose AI use (74 %)</t>
         </is>
       </c>
       <c r="K72" s="7" t="inlineStr">
@@ -18074,7 +18054,7 @@
       <c r="I73" s="7" t="inlineStr"/>
       <c r="J73" s="7" t="inlineStr">
         <is>
-          <t>A1 Clear rules for AI use in assessed work (79 %); A2 Students should always disclose AI use (74 %); T9 Assignments and project descriptions (57 %)</t>
+          <t>T3 Solving or explaining problems step by step (87 %); T4 Exam preparation (86 %); T8 Quiz or exam questions (63 %); T9 Assignments and project descriptions (57 %); T11 Questions on regulations and procedures (61 %); A1 Clear rules for AI use in assessed work (79 %); A2 Students should always disclose AI use (74 %)</t>
         </is>
       </c>
       <c r="K73" s="7" t="inlineStr">
@@ -18615,7 +18595,7 @@
       <c r="I78" s="7" t="inlineStr"/>
       <c r="J78" s="7" t="inlineStr">
         <is>
-          <t>A3 More trust in AI output with visible sources (67 %)</t>
+          <t>T11 Questions on regulations and procedures (61 %); A3 More trust in AI output with visible sources (67 %)</t>
         </is>
       </c>
       <c r="K78" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Rename the evidence column of profile.xlsx to basis
The column lists the basis of each element in the three perspectives
(P1 standards, P2 practice, P3 AI use), as in Annex A of the MS4 report.
README and landing page follow the new name. Content is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -531,7 +531,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MS4 report, Annex A (definitions, mappings, evidence) and Annex G (candidate fields)</t>
+          <t>MS4 report, Annex A (definitions, mappings, basis) and Annex G (candidate fields)</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>evidence</t>
+          <t>basis</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
@@ -8356,7 +8356,7 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>evidence</t>
+          <t>basis</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Revert "Rename the evidence column of profile.xlsx to basis"
This reverts commit 66183cf. The column keeps the name evidence.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -531,7 +531,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MS4 report, Annex A (definitions, mappings, basis) and Annex G (candidate fields)</t>
+          <t>MS4 report, Annex A (definitions, mappings, evidence) and Annex G (candidate fields)</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>basis</t>
+          <t>evidence</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
@@ -8356,7 +8356,7 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>basis</t>
+          <t>evidence</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Corrections from the full proofread of the MS10 report
profile.xlsx: evidence of X31, X10, X19, X22, R09 and R04 corrected
against the candidate-field data, frequency of offering (D01) marked
not recommended, P1 marks of four candidate fields with approximate
hooks set to partial. Vocabulary: definition of
generating-submitted-code covers (part of) the submitted work.
Elements, tiers, schema and shapes are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -4737,7 +4737,7 @@
       </c>
       <c r="S43" s="4" t="inlineStr">
         <is>
-          <t>Skills #42</t>
+          <t>Skills #42 (partly)</t>
         </is>
       </c>
     </row>
@@ -4829,7 +4829,7 @@
       </c>
       <c r="R44" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓4–5 · P2 n.m. · P3 –</t>
+          <t>P1 ✓4 (+1 hook) · P2 n.m. · P3 –</t>
         </is>
       </c>
       <c r="S44" s="4" t="inlineStr">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="R48" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 coordinator 6/10; WP4 Md 4, 55 %, ✘ · P3 –</t>
+          <t>P1 ✓4 · P2 coordinator 6/10; WP4 Md 4, 55 %, ✘ · P3 –</t>
         </is>
       </c>
       <c r="S48" s="4" t="inlineStr">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="R49" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓1 (ECTS Guide, learning agreement for work placements) · P2 n.m. · P3 –</t>
+          <t>P1 ✓1 (ECTS guide, learning agreement for work placements) · P2 n.m. · P3 –</t>
         </is>
       </c>
       <c r="S49" s="4" t="inlineStr">
@@ -5993,7 +5993,7 @@
       </c>
       <c r="R56" s="4" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 n.m. (field at 1/10 partners); named as missing in WP4 · P3 T11; MyAI University</t>
+          <t>P1 ✓1 (ECTS guide) · P2 n.m. (field at 1/10 partners); named as missing in WP4 · P3 T11; MyAI University</t>
         </is>
       </c>
       <c r="S56" s="4" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="R59" s="4" t="inlineStr">
         <is>
-          <t>P1 hook · P2 n.m. · P3 –; MyAI University</t>
+          <t>P1 ✓1 (schema.org) · P2 n.m. · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S59" s="4" t="inlineStr">
@@ -7254,7 +7254,7 @@
       </c>
       <c r="R69" s="5" t="inlineStr">
         <is>
-          <t>P1 ✓5 · P2 currency 2/10 (+2); manual version/date ●3/10, ◐5/10; WP4 Md 4, 64 %, ✘ · P3 A3; MyAI University</t>
+          <t>P1 ✓5 (date group) · P2 currency 2/10 (+2); manual version/date ●3/10, ◐5/10; WP4 Md 4, 64 %, ✘ · P3 T11, A3; MyAI University</t>
         </is>
       </c>
       <c r="S69" s="5" t="inlineStr">
@@ -7739,7 +7739,7 @@
       </c>
       <c r="R74" s="5" t="inlineStr">
         <is>
-          <t>P1 hook · P2 n.m. · P3 A3; design input</t>
+          <t>P1 ✓1 (schema.org) · P2 n.m. · P3 A3; design input</t>
         </is>
       </c>
       <c r="S74" s="5" t="inlineStr">
@@ -9390,7 +9390,7 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Mapped to the linked offering</t>
+          <t>Not recommended (derivable from the linked offering)</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
@@ -10945,7 +10945,7 @@
       <c r="R9" s="7" t="inlineStr"/>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>○</t>
+          <t>◐</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="S15" s="7" t="inlineStr">
         <is>
-          <t>○</t>
+          <t>◐</t>
         </is>
       </c>
       <c r="T15" s="7" t="inlineStr">
@@ -13996,7 +13996,7 @@
       <c r="R36" s="7" t="inlineStr"/>
       <c r="S36" s="7" t="inlineStr">
         <is>
-          <t>○</t>
+          <t>◐</t>
         </is>
       </c>
       <c r="T36" s="7" t="inlineStr">
@@ -14422,7 +14422,7 @@
       <c r="R40" s="7" t="inlineStr"/>
       <c r="S40" s="7" t="inlineStr">
         <is>
-          <t>○</t>
+          <t>◐</t>
         </is>
       </c>
       <c r="T40" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Corrections from the v16 read-through
- Precedence rule 3: exclusions matter under permitted-with-disclosure and
  required; no longer forbidden under other levels (matches the full example)
- Gate: all referenced components and outcomes must be met
- Conventions: disclosure scope and input of course materials listed as closed
- Full example: AI conditions of the mini-projects and exercises repeat the
  course rule on course materials (360 triples)
- Element list: A11 definition, R14 ECTS note, D06/D07 wording, F03 tier

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -3411,7 +3411,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Default rules for AI use in the unit: permission level, permitted/excluded purposes, disclosure, verification, interaction-mode hint, approved tools, note, institutional policy link.</t>
+          <t>Default rules for AI use in the unit: permission level, permitted/excluded purposes, disclosure and disclosure scope, verification, interaction-mode hint, input of course materials, protected outcomes and mastery gate, approved tools, note, institutional policy link.</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -8199,7 +8199,7 @@
       </c>
       <c r="M79" s="5" t="inlineStr">
         <is>
-          <t>≈ national language + English required</t>
+          <t>≈ national language + English recommended</t>
         </is>
       </c>
       <c r="N79" s="5" t="inlineStr">
@@ -9500,7 +9500,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Merged into R10</t>
+          <t>Covered by R10</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -9522,7 +9522,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Merged into X30</t>
+          <t>Covered by X30</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -10387,7 +10387,7 @@
       </c>
       <c r="P4" s="7" t="inlineStr">
         <is>
-          <t>Core (identification)</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Q4" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Evidence marks aligned with the field table; two not-recommended candidates documented (D26, D27)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -755,7 +755,7 @@
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓5 · P2 6/10; WP4 Md 4, 73 %, ✘ · P3 –</t>
+          <t>P1 ✓5 · P2 6/10; WP4 Md 4, 73 %, ✘ · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="R24" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 n.m. (field present only in one blank template); named as missing in WP4 · P3 T5, T7, T9; design input</t>
+          <t>P1 hook · P2 n.m. (field present only in one blank template); named as missing in WP4 · P3 T5, T7, T9; design input</t>
         </is>
       </c>
       <c r="S24" s="3" t="inlineStr">
@@ -3277,7 +3277,7 @@
       </c>
       <c r="R28" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 n.m. (no field in any partner document) · P3 T2, T3, T5, T8; design input</t>
+          <t>P1 hook · P2 n.m. (no field in any partner document) · P3 T2, T3, T5, T8; design input</t>
         </is>
       </c>
       <c r="S28" s="3" t="inlineStr">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="R32" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 n.m.; exam settings implicit in assessment methods · P3 T4, A1; Corbin et al., 2025; Verbeken et al., 2026 (supervised setting rated low risk in an institutional rubric)</t>
+          <t>P1 hook · P2 n.m.; exam settings implicit in assessment methods · P3 T4, A1; Corbin et al., 2025; Verbeken et al., 2026 (supervised setting rated low risk in an institutional rubric)</t>
         </is>
       </c>
       <c r="S32" s="3" t="inlineStr">
@@ -4247,7 +4247,7 @@
       </c>
       <c r="R38" s="4" t="inlineStr">
         <is>
-          <t>P1 ✓3 (as subject) · P2 n.m. · P3 –</t>
+          <t>P1 ✓3 (as subject) · P2 n.m. · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S38" s="4" t="inlineStr">
@@ -5896,7 +5896,7 @@
       </c>
       <c r="R55" s="4" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 n.m. · P3 –; MyAI University</t>
+          <t>P1 hook · P2 n.m. · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S55" s="4" t="inlineStr">
@@ -6090,7 +6090,7 @@
       </c>
       <c r="R57" s="4" t="inlineStr">
         <is>
-          <t>P1 n/a · P2 n.m. · P3 –</t>
+          <t>P1 n/a · P2 n.m. · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S57" s="4" t="inlineStr">
@@ -7157,7 +7157,7 @@
       </c>
       <c r="R68" s="5" t="inlineStr">
         <is>
-          <t>P1 ✓5 (date group) · P2 currency 2/10 (+2); WP4 Md 4, 64 %, ✘ · P3 T11, A3; MyAI University</t>
+          <t>P1 ✓5 (date group: created, modified or issued) · P2 currency 2/10 (+2); WP4 Md 4, 64 %, ✘ · P3 T11, A3; MyAI University</t>
         </is>
       </c>
       <c r="S68" s="5" t="inlineStr">
@@ -7254,7 +7254,7 @@
       </c>
       <c r="R69" s="5" t="inlineStr">
         <is>
-          <t>P1 ✓5 (date group) · P2 currency 2/10 (+2); manual version/date ●3/10, ◐5/10; WP4 Md 4, 64 %, ✘ · P3 T11, A3; MyAI University</t>
+          <t>P1 ✓5 (date group: created, modified or issued) · P2 currency 2/10 (+2); manual version/date ●3/10, ◐5/10; WP4 Md 4, 64 %, ✘ · P3 T11, A3; MyAI University</t>
         </is>
       </c>
       <c r="S69" s="5" t="inlineStr">
@@ -7642,7 +7642,7 @@
       </c>
       <c r="R73" s="5" t="inlineStr">
         <is>
-          <t>P1 ✓1 (dcterms:source) · P2 n.m. · P3 –</t>
+          <t>P1 ✓1 (dcterms:source) · P2 n.m. · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S73" s="5" t="inlineStr">
@@ -7933,7 +7933,7 @@
       </c>
       <c r="R76" s="5" t="inlineStr">
         <is>
-          <t>P1 hook · P2 n.m. · P3 –</t>
+          <t>P1 hook · P2 n.m. · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S76" s="5" t="inlineStr">
@@ -8030,7 +8030,7 @@
       </c>
       <c r="R77" s="5" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 n.m. · P3 –</t>
+          <t>P1 ✓3 · P2 n.m. · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S77" s="5" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="R78" s="5" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 n.m. · P3 –</t>
+          <t>P1 ✓2 · P2 n.m. · P3 –; MyAI University</t>
         </is>
       </c>
       <c r="S78" s="5" t="inlineStr">
@@ -9346,7 +9346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9924,6 +9924,50 @@
       <c r="D26" s="7" t="inlineStr">
         <is>
           <t>Offered by schema.org for the licence of the structured data, whatever vocabularies it combines. Decided with the review of the profile (Section 10); openly published records should state it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>D26</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Derived from / adaptation of another unit</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Not recommended</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Offered by schema.org and LRMI. Covered by the version relations of the record (R13).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>D27</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Spatial or temporal coverage of the content</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Not recommended</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Offered by LOM, schema.org and Dublin Core. Not meaningful for course units.</t>
         </is>
       </c>
     </row>
@@ -9946,7 +9990,7 @@
     <col width="11.2" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="8.800000000000001" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24.8" customWidth="1" min="6" max="6"/>
     <col width="27.2" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="36" customWidth="1" min="9" max="9"/>
@@ -10136,7 +10180,11 @@
       </c>
       <c r="I2" s="7" t="inlineStr"/>
       <c r="J2" s="7" t="inlineStr"/>
-      <c r="K2" s="7" t="inlineStr"/>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>MyAI University</t>
+        </is>
+      </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
           <t>3/3 yes</t>
@@ -10194,7 +10242,7 @@
       </c>
       <c r="W2" s="7" t="inlineStr">
         <is>
-          <t>·</t>
+          <t>◐</t>
         </is>
       </c>
       <c r="X2" s="7" t="inlineStr">
@@ -10950,7 +10998,7 @@
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="U9" s="7" t="inlineStr">
@@ -12062,7 +12110,7 @@
       </c>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="U19" s="7" t="inlineStr">
@@ -13884,7 +13932,7 @@
       </c>
       <c r="T35" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="U35" s="7" t="inlineStr">
@@ -14178,7 +14226,11 @@
       </c>
       <c r="I38" s="7" t="inlineStr"/>
       <c r="J38" s="7" t="inlineStr"/>
-      <c r="K38" s="7" t="inlineStr"/>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>MyAI University</t>
+        </is>
+      </c>
       <c r="L38" s="7" t="inlineStr">
         <is>
           <t>0/3 yes</t>
@@ -14228,7 +14280,7 @@
       </c>
       <c r="W38" s="7" t="inlineStr">
         <is>
-          <t>·</t>
+          <t>◐</t>
         </is>
       </c>
       <c r="X38" s="7" t="inlineStr">
@@ -14756,7 +14808,7 @@
       </c>
       <c r="T43" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="U43" s="7" t="inlineStr">
@@ -16515,7 +16567,11 @@
       </c>
       <c r="I59" s="7" t="inlineStr"/>
       <c r="J59" s="7" t="inlineStr"/>
-      <c r="K59" s="7" t="inlineStr"/>
+      <c r="K59" s="7" t="inlineStr">
+        <is>
+          <t>MyAI University</t>
+        </is>
+      </c>
       <c r="L59" s="7" t="inlineStr">
         <is>
           <t>–</t>
@@ -16569,7 +16625,7 @@
       </c>
       <c r="W59" s="7" t="inlineStr">
         <is>
-          <t>·</t>
+          <t>◐</t>
         </is>
       </c>
       <c r="X59" s="7" t="inlineStr">
@@ -16753,7 +16809,7 @@
       </c>
       <c r="Q61" s="7" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>D26</t>
         </is>
       </c>
       <c r="R61" s="7" t="inlineStr">
@@ -16860,7 +16916,7 @@
       </c>
       <c r="Q62" s="7" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>D27</t>
         </is>
       </c>
       <c r="R62" s="7" t="inlineStr">
@@ -17586,7 +17642,7 @@
       <c r="E69" s="7" t="inlineStr"/>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>hook (ECTS: alignment in prose)</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
@@ -17643,7 +17699,7 @@
       <c r="R69" s="7" t="inlineStr"/>
       <c r="S69" s="7" t="inlineStr">
         <is>
-          <t>○</t>
+          <t>◐</t>
         </is>
       </c>
       <c r="T69" s="7" t="inlineStr">
@@ -17816,7 +17872,7 @@
       <c r="E71" s="7" t="inlineStr"/>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>hook (LOM 5.10 free text)</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -17869,7 +17925,7 @@
       <c r="R71" s="7" t="inlineStr"/>
       <c r="S71" s="7" t="inlineStr">
         <is>
-          <t>○</t>
+          <t>◐</t>
         </is>
       </c>
       <c r="T71" s="7" t="inlineStr">
@@ -18915,7 +18971,11 @@
       </c>
       <c r="I81" s="7" t="inlineStr"/>
       <c r="J81" s="7" t="inlineStr"/>
-      <c r="K81" s="7" t="inlineStr"/>
+      <c r="K81" s="7" t="inlineStr">
+        <is>
+          <t>MyAI University</t>
+        </is>
+      </c>
       <c r="L81" s="7" t="inlineStr">
         <is>
           <t>0/3 yes</t>
@@ -18965,7 +19025,7 @@
       </c>
       <c r="W81" s="7" t="inlineStr">
         <is>
-          <t>·</t>
+          <t>◐</t>
         </is>
       </c>
       <c r="X81" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Corrections from the final read-through
- Precedence rule 10: before a gate is met, no AI use in the scope of the
  policy, and less specific rules do not apply in its place
- Conventions and term definitions aligned with the report (validation
  groups, approved tools, ownership of schemes to be decided in the review)
- Element list: evidence notes (R14 bilingual versions not linked, D26 reason,
  MyAI University area names); validator notes list the rules left to a
  semantic validator consistently

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -2598,7 +2598,7 @@
       </c>
       <c r="R21" s="3" t="inlineStr">
         <is>
-          <t>P1 hook · P2 manual ●2/10, ◐4/10 (five different outcome models in use) · P3 T10; design input</t>
+          <t>P1 hook · P2 manual ●2/10, ◐4/10 (at least five different outcome models in use) · P3 T10; design input</t>
         </is>
       </c>
       <c r="S21" s="3" t="inlineStr">
@@ -4446,7 +4446,7 @@
       </c>
       <c r="S40" s="4" t="inlineStr">
         <is>
-          <t>LOs #16, #17; Skills #40, #41, #42 (R); §7 "AI competence taught"</t>
+          <t>LOs &amp; competencies #16, #17; Skills #40, #41, #42 (R); §7 "AI competence taught"</t>
         </is>
       </c>
     </row>
@@ -6871,7 +6871,7 @@
       </c>
       <c r="S65" s="4" t="inlineStr">
         <is>
-          <t>Format &amp; delivery #18, #22; Workload #29; MyAI University framework §4.3 "form of participation"</t>
+          <t>Format &amp; delivery #18, #22; Workload &amp; time #29; MyAI University framework §4.3 "form of participation"</t>
         </is>
       </c>
     </row>
@@ -8224,7 +8224,7 @@
       </c>
       <c r="R79" s="5" t="inlineStr">
         <is>
-          <t>P1 ✓1 (schema.org) · P2 bilingual versions at 2/10 (manual review) · P3 –</t>
+          <t>P1 ✓1 (schema.org) · P2 0/10 (bilingual versions at 2/10, not linked) · P3 –</t>
         </is>
       </c>
       <c r="S79" s="5" t="inlineStr">
@@ -9945,7 +9945,7 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Offered by schema.org and LRMI. Covered by the version relations of the record (R13).</t>
+          <t>Offered by schema.org and LRMI. Rarely needed for course units. Where relevant, it can be stated in the content description (C06).</t>
         </is>
       </c>
     </row>
@@ -16814,7 +16814,7 @@
       </c>
       <c r="R61" s="7" t="inlineStr">
         <is>
-          <t>isBasedOnUrl, exampleOfWork; covered by version relations</t>
+          <t>isBasedOnUrl, exampleOfWork; rarely needed for course units</t>
         </is>
       </c>
       <c r="S61" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Consistency fixes from the read-through of the extensions
- course-default: the rule that would apply without the gated policy (usually
  the course rule), only on assessment conditions; vocabulary page and rule 10
  regenerated
- Precedence rules: rule 2 points to the gate, rule 10 covers tools that cannot
  check the gate and gates on course-level policies; excludedPurpose wording
- Shapes: value checks also reach a rule before the gate without @type
  (new test, 69 in total)
- Full example: the rule before the gate repeats the course rule on course
  materials (367 triples); schema description updated
- Element list: class definition, A11 vocabulary, D04, D19, D23 references

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -3421,7 +3421,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>Annex C (euvoc:ai-*)</t>
+          <t>Annex C (euvoc:ai-*, euvoc:before-gate/)</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -9456,7 +9456,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Not recommended</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -9791,7 +9791,7 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Low priority in the requirements; candidate for D2.2/D4.2.</t>
+          <t>Not covered by the requirements of Section 2, and no need found in the evidence. Candidate for D2.2/D4.2.</t>
         </is>
       </c>
     </row>
@@ -10001,7 +10001,7 @@
     <col width="60" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="27.2" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
     <col width="60" customWidth="1" min="18" max="18"/>
     <col width="8" customWidth="1" min="19" max="19"/>
     <col width="10.4" customWidth="1" min="20" max="20"/>
@@ -17237,7 +17237,7 @@
       </c>
       <c r="Q65" s="7" t="inlineStr">
         <is>
-          <t>A11</t>
+          <t>D23 (linked via A11)</t>
         </is>
       </c>
       <c r="R65" s="7" t="inlineStr">
@@ -18323,11 +18323,7 @@
       </c>
       <c r="I75" s="7" t="inlineStr"/>
       <c r="J75" s="7" t="inlineStr"/>
-      <c r="K75" s="7" t="inlineStr">
-        <is>
-          <t>requirements (optional)</t>
-        </is>
-      </c>
+      <c r="K75" s="7" t="inlineStr"/>
       <c r="L75" s="7" t="inlineStr">
         <is>
           <t>–</t>
@@ -18377,7 +18373,7 @@
       </c>
       <c r="W75" s="7" t="inlineStr">
         <is>
-          <t>◐</t>
+          <t>·</t>
         </is>
       </c>
       <c r="X75" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Corrections after the review of report v16
- Generation method: human-authored, ai-assisted, ai-assisted-human-reviewed
  (AI-assisted covers extraction, enrichment and drafting; mixed-record rule)
- Core-level example is a separate course (NLP-2040) with its own identifiers;
  new test checks that the examples share no course-unit IRIs (70 tests)
- Precedence rules: evaluation sequence (rule 2), exclusions and overlapping
  purposes (rule 3); approvedTool is an informational list
- Gate: progression gate vs unaided mastery; assessment setting as a coarse
  summary; element definitions (C13, A04, X21, R09)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -1665,7 +1665,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Course-unit learning outcomes as first-class objects: each has an IRI, a short code and a statement (multilingual), ideally in "active verb + object + context" form (ECTS guide).</t>
+          <t>Course-unit learning outcomes as first-class objects: each has a stable identifier, may have a short display code and has a statement (multilingual), ideally in "active verb + object + context" form (ECTS guide).</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -2732,7 +2732,7 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Outcome(s) each assessment component assesses. This is the outcome → assessment side of constructive alignment.</t>
+          <t>Outcome(s) each assessment component assesses. This is the assessment → outcome link of constructive alignment.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Conditions under which an assessment component is completed: supervised or unsupervised, on site or remote, time-limited or open; a neutral description, recorded independently of the AI-use rules and of the assessment AI class (Annex C.8).</t>
+          <t>Conditions under which an assessment component is completed: supervised or unsupervised, on site or remote, time-limited or open; a neutral description, recorded independently of the AI-use rules and of the assessment AI class (Annex C.8). The four values are a coarse summary that combines supervision with location or timing, sufficient for the current use cases. They do not capture each dimension independently.</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -6127,7 +6127,7 @@
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Tuition or participation fees for the offering, or free of charge.</t>
+          <t>Default tuition or participation fees of the unit, or free of charge. Actual fees of a particular offering belong to the offering (§A.4a).</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
@@ -7679,7 +7679,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>How the record was produced. Mandatory.</t>
+          <t>How the record was produced. Mandatory. AI-assisted covers extraction, enrichment and drafting with AI. A record is AI-assisted as soon as any element was extracted, proposed or drafted with AI and kept, and human-reviewed when a person has checked every such element. Approval is recorded separately (R10).</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
@@ -7689,12 +7689,12 @@
       </c>
       <c r="H74" s="5" t="inlineStr">
         <is>
-          <t>euvoc:generation/: human-authored / ai-extracted / ai-extracted-human-reviewed</t>
+          <t>euvoc:generation/: human-authored / ai-assisted / ai-assisted-human-reviewed</t>
         </is>
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>euonair:generationMethod; digitalSourceType (schema.org) for AI-generated or AI-assisted content</t>
+          <t>euonair:generationMethod; digitalSourceType (schema.org, supplementary information on AI-generated or AI-assisted content)</t>
         </is>
       </c>
       <c r="J74" s="5" t="inlineStr">
@@ -9292,7 +9292,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>human-authored · ai-extracted · ai-extracted-human-reviewed</t>
+          <t>human-authored · ai-assisted · ai-assisted-human-reviewed</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -9395,7 +9395,7 @@
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>P1 hook only; P2 2/10 (+1); WP4 Md 3, 36 %. Derived from the offerings (O01), where partners that use it can record it.</t>
+          <t>P1 hook only; P2 2/10 (+1); WP4 Md 3, 36 %. Derived from the dated offerings (O01) where offerings are scheduled. Where a planned frequency (for example annual or biennial) matters before offerings are scheduled, it can be stated in the content description or the access conditions (C06, X22).</t>
         </is>
       </c>
     </row>
@@ -9527,7 +9527,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Year of study is redundant when the semester is given; track Md 4, 64 %, ✘.</t>
+          <t>Year of study follows from the recommended semester where the programme has a defined curriculum calendar. Where it does not, the position is stated in the placement element (X30). track Md 4, 64 %, ✘.</t>
         </is>
       </c>
     </row>
@@ -9967,7 +9967,7 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Offered by LOM, schema.org and Dublin Core. Not meaningful for course units.</t>
+          <t>Offered by LOM, schema.org and Dublin Core. A separate structured field is not required by the current use cases. Regional or historical coverage can be stated in the content description or topics (C06, C07).</t>
         </is>
       </c>
     </row>
@@ -11971,7 +11971,7 @@
       </c>
       <c r="N18" s="7" t="inlineStr">
         <is>
-          <t>6 empirical of 6: Alier2025, BeutlingSpahicBogdanovic2024, Doughty2024, HoLam2026, PardosNam2020, Pereira2024</t>
+          <t>5 empirical of 6: Alier2025, BeutlingSpahicBogdanovic2024, Doughty2024, HoLam2026, PardosNam2020, Pereira2024</t>
         </is>
       </c>
       <c r="O18" s="7" t="inlineStr">
@@ -12197,7 +12197,7 @@
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>5 empirical of 6: AbuSalih2024, HoLam2026, Kazemitabaar2024, Liffiton2023, Liu2024CS50, Pereira2024</t>
+          <t>4 empirical of 6: AbuSalih2024, HoLam2026, Kazemitabaar2024, Liffiton2023, Liu2024CS50, Pereira2024</t>
         </is>
       </c>
       <c r="O20" s="7" t="inlineStr">
@@ -13220,7 +13220,7 @@
       </c>
       <c r="N29" s="7" t="inlineStr">
         <is>
-          <t>17 empirical of 22: AbuSalih2024, Alier2025, BeutlingSpahicBogdanovic2024, ChandrasekaranMago2022, Doughty2024, Duarte2024, Groher2026, Heppner2019, HoLam2026, Humble2025, Jensen2024, Kestin2025, Kolagar2025, Li2022, Liffiton2023, Pereira2024, Perkins2024, Riahi2026, Sajja2023, Shaikh2021, Stanny2016, Verbeken2026</t>
+          <t>16 empirical of 22: AbuSalih2024, Alier2025, BeutlingSpahicBogdanovic2024, ChandrasekaranMago2022, Doughty2024, Duarte2024, Groher2026, Heppner2019, HoLam2026, Humble2025, Jensen2024, Kestin2025, Kolagar2025, Li2022, Liffiton2023, Pereira2024, Perkins2024, Riahi2026, Sajja2023, Shaikh2021, Stanny2016, Verbeken2026</t>
         </is>
       </c>
       <c r="O29" s="7" t="inlineStr">
@@ -17341,7 +17341,7 @@
       </c>
       <c r="N66" s="7" t="inlineStr">
         <is>
-          <t>8 empirical of 9: ChandrasekaranMago2022, Doughty2024, Heppner2019, HoLam2026, Kestin2025, Kolagar2025, Li2022, Shaikh2021, Stanny2016</t>
+          <t>7 empirical of 9: ChandrasekaranMago2022, Doughty2024, Heppner2019, HoLam2026, Kestin2025, Kolagar2025, Li2022, Shaikh2021, Stanny2016</t>
         </is>
       </c>
       <c r="O66" s="7" t="inlineStr">
@@ -17793,7 +17793,7 @@
       </c>
       <c r="N70" s="7" t="inlineStr">
         <is>
-          <t>1 empirical of 1: HoLam2026</t>
+          <t>0 empirical of 1: HoLam2026</t>
         </is>
       </c>
       <c r="O70" s="7" t="inlineStr">
@@ -17844,7 +17844,7 @@
       </c>
       <c r="Y70" s="7" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>◐</t>
         </is>
       </c>
     </row>
@@ -18667,7 +18667,7 @@
       </c>
       <c r="N78" s="7" t="inlineStr">
         <is>
-          <t>2 empirical of 3: HoLam2026, Humble2025, Liu2024CS50</t>
+          <t>1 empirical of 3: HoLam2026, Humble2025, Liu2024CS50</t>
         </is>
       </c>
       <c r="O78" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Documentation wording aligned with report v20 (0.9.2)
Element definitions, conventions and AI-use rules follow the copy-edited
report: cognitive level and competence category stated as closed lists,
expectation codes E1–E4, clearer precedence rules. Vocabularies, context,
schema, shapes and examples are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -852,7 +852,7 @@
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓5 · P2 10/10; WP4 Md 5, 82 %, ✔ · P3 A3; MyAI University</t>
+          <t>P1 ✓5 · P2 10/10; WP4 Md 5, 82 %, ✔ · P3 E3; MyAI University</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓3 · P2 0/10; WP4 Md 5, 82 %, ✔ · P3 T11, A3, A4</t>
+          <t>P1 ✓3 · P2 0/10; WP4 Md 5, 82 %, ✔ · P3 T11, E3, E4</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>P1 ✓4 · P2 8/10; WP4 Md 4, 82 %, ✔ · P3 T1, T2, T3, T4, T5, T6, T8, A3, A4</t>
+          <t>P1 ✓4 · P2 8/10; WP4 Md 4, 82 %, ✔ · P3 T1, T2, T3, T4, T5, T6, T8, E3, E4</t>
         </is>
       </c>
       <c r="S19" s="2" t="inlineStr">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>revised Bloom (default): remember / understand / apply / analyse / evaluate / create; others (SOLO …) allowed via own scheme</t>
+          <t>revised Bloom: remember / understand / apply / analyse / evaluate / create (only these values in profile version 0.9; other schemes such as SOLO deferred to a later version)</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -3471,7 +3471,7 @@
       </c>
       <c r="R30" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 no field in any partner; AI rules found only at assessment level (A12) · P3 T3, T11, A1, A2; all reported institutional policies PDF/web only; design input</t>
+          <t>P1 ✗ · P2 no field in any partner; AI rules found only at assessment level (A12) · P3 T3, T11, E1, E2; all reported institutional policies PDF/web only; design input</t>
         </is>
       </c>
       <c r="S30" s="3" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="R31" s="3" t="inlineStr">
         <is>
-          <t>P1 ✗ · P2 1/10 (permitted aids of individual exams, 7 of 125 module descriptions) · P3 T3, T4, T8, T9, T11, A1, A2; institutional policies cover assessments at 7 of 9; design input</t>
+          <t>P1 ✗ · P2 1/10 (permitted aids of individual exams, 7 of 125 module descriptions) · P3 T3, T4, T8, T9, T11, E1, E2; institutional policies cover assessments at 7 of 9; design input</t>
         </is>
       </c>
       <c r="S31" s="3" t="inlineStr">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="R32" s="3" t="inlineStr">
         <is>
-          <t>P1 hook · P2 n.m.; exam settings implicit in assessment methods · P3 T4, A1; Corbin et al., 2025; Verbeken et al., 2026 (supervised setting rated low risk in an institutional rubric)</t>
+          <t>P1 hook · P2 n.m.; exam settings implicit in assessment methods · P3 T4, E1; Corbin et al., 2025; Verbeken et al., 2026 (supervised setting rated low risk in an institutional rubric)</t>
         </is>
       </c>
       <c r="S32" s="3" t="inlineStr">
@@ -3702,7 +3702,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Licence of the course description, plus optional terms for the materials. Tells AI tools and platforms whether they may ingest and reuse the content. Includes the rights holder and copyright notice (copyrightHolder, copyrightNotice, dcterms:dateCopyrighted; offered by the standards beyond current practice). A11 governs students' use of AI; it does not grant rights to process materials, which depend on the rights in each resource (D24).</t>
+          <t>Licence of the course description, plus optional terms for the materials. Tells AI tools and platforms whether they may ingest and reuse the content. Includes the rights holder and copyright notice (copyrightHolder, copyrightNotice, dcterms:dateCopyrighted; offered by the standards beyond current practice). A11 governs students' use of AI; it does not grant rights to process materials, which depend on the rights in each resource (Annex A.7, D24).</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -7157,7 +7157,7 @@
       </c>
       <c r="R68" s="5" t="inlineStr">
         <is>
-          <t>P1 ✓5 (date group: created, modified or issued) · P2 currency 2/10 (+2); WP4 Md 4, 64 %, ✘ · P3 T11, A3; MyAI University</t>
+          <t>P1 ✓5 (date group: created, modified or issued) · P2 currency 2/10 (+2); WP4 Md 4, 64 %, ✘ · P3 T11, E3; MyAI University</t>
         </is>
       </c>
       <c r="S68" s="5" t="inlineStr">
@@ -7254,7 +7254,7 @@
       </c>
       <c r="R69" s="5" t="inlineStr">
         <is>
-          <t>P1 ✓5 (date group: created, modified or issued) · P2 currency 2/10 (+2); manual version/date ●3/10, ◐5/10; WP4 Md 4, 64 %, ✘ · P3 T11, A3; MyAI University</t>
+          <t>P1 ✓5 (date group: created, modified or issued) · P2 currency 2/10 (+2); manual version/date ●3/10, ◐5/10; WP4 Md 4, 64 %, ✘ · P3 T11, E3; MyAI University</t>
         </is>
       </c>
       <c r="S69" s="5" t="inlineStr">
@@ -7351,7 +7351,7 @@
       </c>
       <c r="R70" s="5" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 as R04; WP4 Md 4, 64 %, ✘ · P3 A3; MyAI University</t>
+          <t>P1 ✓2 · P2 as R04; WP4 Md 4, 64 %, ✘ · P3 E3; MyAI University</t>
         </is>
       </c>
       <c r="S70" s="5" t="inlineStr">
@@ -7448,7 +7448,7 @@
       </c>
       <c r="R71" s="5" t="inlineStr">
         <is>
-          <t>P1 ✓2 · P2 n.m.; WP4 Md 4, 64 %, ✘ · P3 T11, A3; MyAI University</t>
+          <t>P1 ✓2 · P2 n.m.; WP4 Md 4, 64 %, ✘ · P3 T11, E3; MyAI University</t>
         </is>
       </c>
       <c r="S71" s="5" t="inlineStr">
@@ -7739,7 +7739,7 @@
       </c>
       <c r="R74" s="5" t="inlineStr">
         <is>
-          <t>P1 ✓1 (schema.org) · P2 n.m. · P3 A3; design input</t>
+          <t>P1 ✓1 (schema.org) · P2 n.m. · P3 E3; design input</t>
         </is>
       </c>
       <c r="S74" s="5" t="inlineStr">
@@ -9161,7 +9161,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>partner practice (individual/group recorded per element)</t>
+          <t>the partners' practice (individual/group recorded per element)</t>
         </is>
       </c>
     </row>
@@ -9212,7 +9212,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>revised Bloom (Anderson &amp; Krathwohl, 2001); default only</t>
+          <t>revised Bloom (Anderson &amp; Krathwohl, 2001); the only accepted values in profile version 0.9, other schemes such as SOLO deferred to a later version</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrections after the review of report v20 (0.9.3)
Workbook expectation codes E1–E4 and F53 inference note; descriptive
shapes for A13, X32 and O01 properties named in Annex A; euonair:
sub-properties of X30 and X19 listed as terms; accessibility summary as
language-tagged string; vocabulary page states the status of each scheme;
citation and CITATION.cff; profile/0.9/ described as following the
current 0.9.x release. Value lists, context and JSON Schema unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -559,7 +559,7 @@
     <col width="60" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
     <col width="15.2" customWidth="1" min="10" max="10"/>
-    <col width="58.40000000000001" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
     <col width="19.2" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
     <col width="44" customWidth="1" min="14" max="14"/>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Default rules for AI use in the unit: permission level, permitted/excluded purposes, disclosure and disclosure scope, verification, interaction-mode hint, input of course materials, protected outcomes, mastery gate and the rule before it, approved tools, note, institutional policy link.</t>
+          <t>Default rules for AI use in the unit: permission level, permitted/excluded purposes, disclosure and disclosure scope, verification, interaction-mode hint, input of course materials, protected outcomes, gate and the rule before it, approved tools, note, institutional policy link.</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -3707,7 +3707,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>IRI 0..1 (license, SPDX/CC); IRI 0..1 (usageInfo)</t>
+          <t>IRI 0..1 (license, SPDX/CC); IRI 0..1 (usageInfo); Organization/Person 0..1 (copyrightHolder); Text 0..1 (copyrightNotice); Date 0..1 (dcterms:dateCopyrighted)</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -3717,7 +3717,7 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>license, usageInfo</t>
+          <t>license, usageInfo, copyrightHolder, copyrightNotice, dcterms:dateCopyrighted</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
@@ -3727,12 +3727,12 @@
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>schema:license schema:usageInfo</t>
+          <t>schema:license schema:usageInfo schema:copyrightHolder schema:copyrightNotice dcterms:dateCopyrighted</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>0..1 0..1</t>
+          <t>0..1 0..1 0..1 0..1 0..1</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>ProgrammePlacement 0..* {programme Ref, obligation Concept, recommendedSemester int, track Text}</t>
+          <t>ProgrammePlacement 0..* {programme Ref, obligation Concept, recommendedSemester int, track Text} (sub-properties in the euonair: namespace)</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
@@ -5938,7 +5938,7 @@
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>euonair:RecognitionDecision 0..* {equivalentUnit Ref, decidedBy, date}</t>
+          <t>euonair:RecognitionDecision 0..* {equivalentUnit Ref, decidedBy Text, decisionDate Date} (sub-properties in the euonair: namespace)</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
@@ -6821,7 +6821,7 @@
       </c>
       <c r="I65" s="4" t="inlineStr">
         <is>
-          <t>euonair:plannedMode (≈ courseMode, which schema.org defines on CourseInstance), euonair:synchronicity, euonair:pace</t>
+          <t>euonair:plannedMode, euonair:synchronicity, euonair:pace (≈ courseMode for the planned mode, which schema.org defines on CourseInstance)</t>
         </is>
       </c>
       <c r="J65" s="4" t="inlineStr">
@@ -6831,7 +6831,7 @@
       </c>
       <c r="K65" s="4" t="inlineStr">
         <is>
-          <t>euonair:plannedMode</t>
+          <t>euonair:plannedMode euonair:synchronicity euonair:pace</t>
         </is>
       </c>
       <c r="L65" s="4" t="inlineStr">
@@ -8254,8 +8254,8 @@
     <col width="32" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="17.6" customWidth="1" min="8" max="8"/>
-    <col width="55.2" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
     <col width="11.2" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
     <col width="8.800000000000001" customWidth="1" min="12" max="12"/>
@@ -8393,22 +8393,22 @@
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>One node per offering: academic term, start/end date, duration, language override.</t>
+          <t>One node per offering: academic term, start/end date, duration, language override, actual mode of delivery and synchronicity.</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>CourseInstance 0..* {academicTerm, startDate, endDate, duration, inLanguage}</t>
+          <t>CourseInstance 0..* {academicTerm, startDate, endDate, duration, inLanguage, courseMode, synchronicity}</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>ISO 8601</t>
+          <t>ISO 8601; euvoc:synchronicity/</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>hasCourseInstance; startDate, endDate, duration, euonair:academicTerm</t>
+          <t>hasCourseInstance; startDate, endDate, duration, courseMode, euonair:academicTerm, euonair:synchronicity</t>
         </is>
       </c>
       <c r="J2" s="6" t="inlineStr">
@@ -8418,7 +8418,7 @@
       </c>
       <c r="K2" s="6" t="inlineStr">
         <is>
-          <t>schema:hasCourseInstance schema:startDate schema:endDate schema:duration euonair:academicTerm</t>
+          <t>schema:hasCourseInstance schema:startDate schema:endDate schema:duration schema:courseMode euonair:academicTerm euonair:synchronicity</t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
@@ -9527,7 +9527,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Year of study follows from the recommended semester where the programme has a defined curriculum calendar. Where it does not, the position is stated in the placement element (X30). track Md 4, 64 %, ✘.</t>
+          <t>Year of study follows from the recommended semester where the programme has a defined curriculum calendar. Where it does not, the position is stated in the placement element (X30). Track: Md 4, 64 %, ✘.</t>
         </is>
       </c>
     </row>
@@ -10405,7 +10405,7 @@
       <c r="I4" s="7" t="inlineStr"/>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>A3 More trust in AI output with visible sources (67 %)</t>
+          <t>E3 More trust in AI output with visible sources (67 %)</t>
         </is>
       </c>
       <c r="K4" s="7" t="inlineStr">
@@ -10625,7 +10625,7 @@
       <c r="I6" s="7" t="inlineStr"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>T11 Questions on regulations and procedures (61 %); A3 More trust in AI output with visible sources (67 %); A4 Course-specific documents given to AI tools by hand (42 %)</t>
+          <t>T11 Questions on regulations and procedures (61 %); E3 More trust in AI output with visible sources (67 %); E4 Course-specific documents given to AI tools by hand (42 %)</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr"/>
@@ -12637,7 +12637,7 @@
       <c r="I24" s="7" t="inlineStr"/>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T3 Solving or explaining problems step by step (87 %); T4 Exam preparation (86 %); T5 Personalised exercise and learning recommendations within a course (65 %); T6 Language learning or translation support (78 %); T8 Quiz or exam questions (63 %); A3 More trust in AI output with visible sources (67 %); A4 Course-specific documents given to AI tools by hand (42 %)</t>
+          <t>T1 Summarising or simplifying reading material (92 %); T2 Explanations of concepts (AI as tutor) (88 %); T3 Solving or explaining problems step by step (87 %); T4 Exam preparation (86 %); T5 Personalised exercise and learning recommendations within a course (65 %); T6 Language learning or translation support (78 %); T8 Quiz or exam questions (63 %); E3 More trust in AI output with visible sources (67 %); E4 Course-specific documents given to AI tools by hand (42 %)</t>
         </is>
       </c>
       <c r="K24" s="7" t="inlineStr"/>
@@ -16021,7 +16021,7 @@
       <c r="I54" s="7" t="inlineStr"/>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>A3 More trust in AI output with visible sources (67 %)</t>
+          <t>E3 More trust in AI output with visible sources (67 %)</t>
         </is>
       </c>
       <c r="K54" s="7" t="inlineStr">
@@ -16061,7 +16061,7 @@
       </c>
       <c r="R54" s="7" t="inlineStr">
         <is>
-          <t>schema:digitalSourceType</t>
+          <t>schema:digitalSourceType. The E3 link is an inference: for descriptions produced with AI, how a record was produced is part of the visible source information (Table 5 note).</t>
         </is>
       </c>
       <c r="S54" s="7" t="inlineStr">
@@ -17999,7 +17999,7 @@
       <c r="I72" s="7" t="inlineStr"/>
       <c r="J72" s="7" t="inlineStr">
         <is>
-          <t>T3 Solving or explaining problems step by step (87 %); T11 Questions on regulations and procedures (61 %); A1 Clear rules for AI use in assessed work (79 %); A2 Students should always disclose AI use (74 %)</t>
+          <t>T3 Solving or explaining problems step by step (87 %); T11 Questions on regulations and procedures (61 %); E1 Clear rules for AI use in assessed work (79 %); E2 Students should always disclose AI use (74 %)</t>
         </is>
       </c>
       <c r="K72" s="7" t="inlineStr">
@@ -18110,7 +18110,7 @@
       <c r="I73" s="7" t="inlineStr"/>
       <c r="J73" s="7" t="inlineStr">
         <is>
-          <t>T3 Solving or explaining problems step by step (87 %); T4 Exam preparation (86 %); T8 Quiz or exam questions (63 %); T9 Assignments and project descriptions (57 %); T11 Questions on regulations and procedures (61 %); A1 Clear rules for AI use in assessed work (79 %); A2 Students should always disclose AI use (74 %)</t>
+          <t>T3 Solving or explaining problems step by step (87 %); T4 Exam preparation (86 %); T8 Quiz or exam questions (63 %); T9 Assignments and project descriptions (57 %); T11 Questions on regulations and procedures (61 %); E1 Clear rules for AI use in assessed work (79 %); E2 Students should always disclose AI use (74 %)</t>
         </is>
       </c>
       <c r="K73" s="7" t="inlineStr">
@@ -18647,7 +18647,7 @@
       <c r="I78" s="7" t="inlineStr"/>
       <c r="J78" s="7" t="inlineStr">
         <is>
-          <t>T11 Questions on regulations and procedures (61 %); A3 More trust in AI output with visible sources (67 %)</t>
+          <t>T11 Questions on regulations and procedures (61 %); E3 More trust in AI output with visible sources (67 %)</t>
         </is>
       </c>
       <c r="K78" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Decisions on the review of report v20 (0.9.4)
Mini-project AI condition: the team keeps the evaluation and the release
decision (note and assessment criteria). JSON Schema and SHACL require
schemaVersion on the course unit (R02). Element list wording for non-
semester positions, approved translations and accommodations.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profile.xlsx
+++ b/profile.xlsx
@@ -5060,7 +5060,7 @@
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>For each programme that uses the unit: programme, obligation (compulsory / compulsory-elective / elective), recommended semester and optional track.</t>
+          <t>For each programme that uses the unit: programme, obligation (compulsory / compulsory-elective / elective), recommended semester and optional track. Profile version 0.9 records the position in the curriculum only as a recommended semester. Other positions (year, trimester, stage) have no structured representation yet and are stated in the content description (C06).</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -7005,7 +7005,7 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>IRI 1..1</t>
+          <t>IRI 1..1 (dcterms:conformsTo); IRI 1..1 (schemaVersion)</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr">
@@ -7030,7 +7030,7 @@
       </c>
       <c r="L67" s="5" t="inlineStr">
         <is>
-          <t>1..1</t>
+          <t>1..1 1..1</t>
         </is>
       </c>
       <c r="M67" s="5" t="inlineStr">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Links between the original description and its translations, with the language of each version and whether a person or a machine translated it. A machine translation is never the authoritative version.</t>
+          <t>Links between the original description and its translations, with the language of each version and whether a person or a machine translated it. An unreviewed machine translation is not authoritative. A reviewed and approved translation may be an approved language version, and the institution states which version governs if versions disagree.</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
@@ -9527,7 +9527,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Year of study follows from the recommended semester where the programme has a defined curriculum calendar. Where it does not, the position is stated in the placement element (X30). Track: Md 4, 64 %, ✘.</t>
+          <t>Year of study follows from the recommended semester where the programme has a defined curriculum calendar. Where it does not, version 0.9 has no structured representation: the position is stated in the content description (C06), and a structured form is deferred to a later version (X30). Track: Md 4, 64 %, ✘.</t>
         </is>
       </c>
     </row>

</xml_diff>